<commit_message>
Update to braconid traits data
</commit_message>
<xml_diff>
--- a/source_data/Braconidae_traits.xlsx
+++ b/source_data/Braconidae_traits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFBE842A-BE9D-CD40-89DC-A3274CA2564C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D33E7AA-AF5C-8B40-8AAD-E63C5411E56B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28180" windowHeight="17460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,9 @@
     <sheet name="Swedish data" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Swedish data'!$A$1:$E$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Swedish data'!$A$1:$F$41</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="97">
   <si>
     <t>Phytophage-parasitoid</t>
     <phoneticPr fontId="3"/>
@@ -317,13 +317,46 @@
   </si>
   <si>
     <t>Includes Maxfischeriinae</t>
+  </si>
+  <si>
+    <t>Clade</t>
+  </si>
+  <si>
+    <t>Brachistinae</t>
+  </si>
+  <si>
+    <t>Doryctinae</t>
+  </si>
+  <si>
+    <t>Mesostoinae</t>
+  </si>
+  <si>
+    <t>Doryctinae_Monarea</t>
+  </si>
+  <si>
+    <t>Doryctinae_Nervellius</t>
+  </si>
+  <si>
+    <t>Doryctinae_Ontsira</t>
+  </si>
+  <si>
+    <t>Doryctinae_Syngaster</t>
+  </si>
+  <si>
+    <t>Wang &amp; Aparicio (2020)</t>
+  </si>
+  <si>
+    <t>Iqbal et al. (2006)</t>
+  </si>
+  <si>
+    <t>Marsh (1988) [reared from branches infested with cerambycids)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -395,6 +428,18 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -413,10 +458,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -432,7 +478,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -440,8 +485,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Default" xfId="1" xr:uid="{97A9FA61-B53C-564A-BB10-C00C98D42059}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -835,19 +888,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H406"/>
+  <dimension ref="A1:I410"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="47.1640625" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="2" width="15.83203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="31.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="21.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="21.5" style="1" customWidth="1"/>
-    <col min="7" max="7" width="23" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="47.1640625" style="1"/>
+    <col min="3" max="4" width="31.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="22.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="21.5" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23" style="1" customWidth="1"/>
+    <col min="9" max="9" width="50.83203125" style="16" customWidth="1"/>
+    <col min="10" max="16384" width="47.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="8" customFormat="1" ht="15">
+    <row r="1" spans="1:9" s="8" customFormat="1" ht="15">
       <c r="A1" s="9" t="s">
         <v>16</v>
       </c>
@@ -857,43 +911,48 @@
       <c r="C1" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="G1" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="H1" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="I1" s="8" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="8" customFormat="1" ht="15">
-      <c r="A2" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="12" t="s">
+    <row r="2" spans="1:9" s="8" customFormat="1" ht="15">
+      <c r="A2" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="F2" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="10"/>
       <c r="G2" s="10"/>
-      <c r="H2" s="11"/>
-    </row>
-    <row r="3" spans="1:8" ht="13" customHeight="1">
+      <c r="H2" s="10"/>
+    </row>
+    <row r="3" spans="1:9" ht="13" customHeight="1">
       <c r="A3" s="6" t="s">
         <v>17</v>
       </c>
@@ -904,20 +963,23 @@
         <v>22</v>
       </c>
       <c r="D3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="7"/>
-    </row>
-    <row r="4" spans="1:8" ht="13" customHeight="1">
+      <c r="I3" s="15"/>
+    </row>
+    <row r="4" spans="1:9" ht="13" customHeight="1">
       <c r="A4" s="6" t="s">
         <v>17</v>
       </c>
@@ -928,20 +990,23 @@
         <v>23</v>
       </c>
       <c r="D4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="7"/>
-    </row>
-    <row r="5" spans="1:8" ht="14">
+      <c r="I4" s="15"/>
+    </row>
+    <row r="5" spans="1:9" ht="14">
       <c r="A5" s="6" t="s">
         <v>17</v>
       </c>
@@ -952,20 +1017,23 @@
         <v>24</v>
       </c>
       <c r="D5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H5" s="7"/>
-    </row>
-    <row r="6" spans="1:8" ht="14">
+      <c r="I5" s="15"/>
+    </row>
+    <row r="6" spans="1:9" ht="15">
       <c r="A6" s="6" t="s">
         <v>17</v>
       </c>
@@ -976,18 +1044,21 @@
         <v>57</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F6" s="6"/>
+      <c r="F6" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="G6" s="6"/>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="6"/>
+      <c r="I6" s="15" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="14">
+    <row r="7" spans="1:9" ht="14">
       <c r="A7" s="6" t="s">
         <v>17</v>
       </c>
@@ -995,23 +1066,26 @@
         <v>21</v>
       </c>
       <c r="C7" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="E7" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="F7" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="G7" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="H7" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H7" s="7"/>
-    </row>
-    <row r="8" spans="1:8" ht="14">
+      <c r="I7" s="15"/>
+    </row>
+    <row r="8" spans="1:9" ht="15">
       <c r="A8" s="6" t="s">
         <v>17</v>
       </c>
@@ -1019,25 +1093,28 @@
         <v>21</v>
       </c>
       <c r="C8" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="F8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="G8" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="H8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="I8" s="15" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="13" customHeight="1">
+    <row r="9" spans="1:9" ht="13" customHeight="1">
       <c r="A9" s="6" t="s">
         <v>17</v>
       </c>
@@ -1048,20 +1125,23 @@
         <v>25</v>
       </c>
       <c r="D9" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="G9" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="H9" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H9" s="7"/>
-    </row>
-    <row r="10" spans="1:8" ht="13" customHeight="1">
+      <c r="I9" s="15"/>
+    </row>
+    <row r="10" spans="1:9" ht="13" customHeight="1">
       <c r="A10" s="6" t="s">
         <v>17</v>
       </c>
@@ -1072,20 +1152,23 @@
         <v>26</v>
       </c>
       <c r="D10" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="H10" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" spans="1:8" ht="13" customHeight="1">
+      <c r="I10" s="15"/>
+    </row>
+    <row r="11" spans="1:9" ht="13" customHeight="1">
       <c r="A11" s="6" t="s">
         <v>17</v>
       </c>
@@ -1095,21 +1178,24 @@
       <c r="C11" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="G11" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="H11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H11" s="7"/>
-    </row>
-    <row r="12" spans="1:8" ht="13" customHeight="1">
+      <c r="I11" s="15"/>
+    </row>
+    <row r="12" spans="1:9" ht="13" customHeight="1">
       <c r="A12" s="6" t="s">
         <v>17</v>
       </c>
@@ -1119,21 +1205,24 @@
       <c r="C12" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="F12" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="G12" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="H12" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H12" s="7"/>
-    </row>
-    <row r="13" spans="1:8" ht="13" customHeight="1">
+      <c r="I12" s="15"/>
+    </row>
+    <row r="13" spans="1:9" ht="13" customHeight="1">
       <c r="A13" s="6" t="s">
         <v>17</v>
       </c>
@@ -1144,22 +1233,25 @@
         <v>29</v>
       </c>
       <c r="D13" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="G13" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="H13" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="I13" s="15" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="13" customHeight="1">
+    <row r="14" spans="1:9" ht="13" customHeight="1">
       <c r="A14" s="6" t="s">
         <v>17</v>
       </c>
@@ -1167,301 +1259,332 @@
         <v>21</v>
       </c>
       <c r="C14" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="15"/>
+    </row>
+    <row r="15" spans="1:9" ht="13" customHeight="1">
+      <c r="A15" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="I15" s="15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="13" customHeight="1">
+      <c r="A16" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="I16" s="15" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="15">
+      <c r="A17" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="13" customHeight="1">
+      <c r="A18" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="G18" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="H18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="I18" s="15" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="13" customHeight="1">
-      <c r="A15" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="6" t="s">
+    <row r="19" spans="1:9" ht="13" customHeight="1">
+      <c r="A19" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E19" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F19" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="7"/>
-    </row>
-    <row r="16" spans="1:8" ht="14">
-      <c r="A16" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="6" t="s">
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="15"/>
+    </row>
+    <row r="20" spans="1:9" ht="15">
+      <c r="A20" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D20" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F20" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="G20" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="H20" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="I20" s="15" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="13" customHeight="1">
-      <c r="A17" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="6" t="s">
+    <row r="21" spans="1:9" ht="13" customHeight="1">
+      <c r="A21" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D21" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E21" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="F21" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="G21" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="H21" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H17" s="7"/>
-    </row>
-    <row r="18" spans="1:8" ht="13" customHeight="1">
-      <c r="A18" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="6" t="s">
+      <c r="I21" s="15"/>
+    </row>
+    <row r="22" spans="1:9" ht="13" customHeight="1">
+      <c r="A22" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D22" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="F22" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="G22" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="H22" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="7"/>
-    </row>
-    <row r="19" spans="1:8" ht="13" customHeight="1">
-      <c r="A19" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C19" s="6" t="s">
+      <c r="I22" s="15"/>
+    </row>
+    <row r="23" spans="1:9" ht="13" customHeight="1">
+      <c r="A23" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D23" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="F23" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="G23" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G19" s="6" t="s">
+      <c r="H23" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H19" s="7"/>
-    </row>
-    <row r="20" spans="1:8" ht="13" customHeight="1">
-      <c r="A20" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" s="6" t="s">
+      <c r="I23" s="15"/>
+    </row>
+    <row r="24" spans="1:9" ht="13" customHeight="1">
+      <c r="A24" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D24" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E24" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="F24" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="G24" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G20" s="6" t="s">
+      <c r="H24" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="I24" s="15" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="13" customHeight="1">
-      <c r="A21" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="6" t="s">
+    <row r="25" spans="1:9" ht="13" customHeight="1">
+      <c r="A25" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D25" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E25" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="G25" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G21" s="6" t="s">
+      <c r="H25" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H21" s="7"/>
-    </row>
-    <row r="22" spans="1:8" ht="13" customHeight="1">
-      <c r="A22" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="6" t="s">
+      <c r="I25" s="15"/>
+    </row>
+    <row r="26" spans="1:9" ht="13" customHeight="1">
+      <c r="A26" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="7"/>
-    </row>
-    <row r="23" spans="1:8" ht="13" customHeight="1">
-      <c r="A23" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="H23" s="7"/>
-    </row>
-    <row r="24" spans="1:8" ht="13" customHeight="1">
-      <c r="A24" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="7" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="13" customHeight="1">
-      <c r="A25" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="7"/>
-    </row>
-    <row r="26" spans="1:8" ht="13" customHeight="1">
-      <c r="A26" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>84</v>
-      </c>
       <c r="D26" s="6" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F26" s="6"/>
+      <c r="F26" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="G26" s="6"/>
-      <c r="H26" s="7" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="13" customHeight="1">
+      <c r="H26" s="6"/>
+      <c r="I26" s="15"/>
+    </row>
+    <row r="27" spans="1:9" ht="13" customHeight="1">
       <c r="A27" s="6" t="s">
         <v>17</v>
       </c>
@@ -1469,39 +1592,51 @@
         <v>21</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="7"/>
-    </row>
-    <row r="28" spans="1:8" ht="13" customHeight="1">
+        <v>19</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I27" s="15"/>
+    </row>
+    <row r="28" spans="1:9" ht="13" customHeight="1">
       <c r="A28" s="6" t="s">
-        <v>17</v>
+        <v>81</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>53</v>
+        <v>82</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F28" s="6"/>
+      <c r="F28" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="G28" s="6"/>
-      <c r="H28" s="7"/>
-    </row>
-    <row r="29" spans="1:8" ht="13" customHeight="1">
+      <c r="H28" s="6"/>
+      <c r="I28" s="15" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="13" customHeight="1">
       <c r="A29" s="6" t="s">
         <v>17</v>
       </c>
@@ -1509,888 +1644,1025 @@
         <v>21</v>
       </c>
       <c r="C29" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="15"/>
+    </row>
+    <row r="30" spans="1:9" ht="13" customHeight="1">
+      <c r="A30" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+      <c r="I30" s="15" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="13" customHeight="1">
+      <c r="A31" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="15"/>
+    </row>
+    <row r="32" spans="1:9" ht="13" customHeight="1">
+      <c r="A32" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="15"/>
+    </row>
+    <row r="33" spans="1:9" ht="13" customHeight="1">
+      <c r="A33" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D33" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E33" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="F33" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="G33" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G29" s="6" t="s">
+      <c r="H33" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H29" s="7"/>
-    </row>
-    <row r="30" spans="1:8" ht="13" customHeight="1">
-      <c r="A30" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C30" s="7" t="s">
+      <c r="I33" s="15"/>
+    </row>
+    <row r="34" spans="1:9" ht="13" customHeight="1">
+      <c r="A34" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C34" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D34" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E34" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="F34" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="G34" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="G30" s="7" t="s">
+      <c r="H34" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H30" s="7" t="s">
+      <c r="I34" s="15" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="13" customHeight="1">
-      <c r="A31" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C31" s="6" t="s">
+    <row r="35" spans="1:9" ht="13" customHeight="1">
+      <c r="A35" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C35" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D35" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E35" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="F35" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F31" s="6" t="s">
+      <c r="G35" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G31" s="6" t="s">
+      <c r="H35" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H31" s="7"/>
-    </row>
-    <row r="32" spans="1:8" ht="13" customHeight="1">
-      <c r="A32" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C32" s="6" t="s">
+      <c r="I35" s="15"/>
+    </row>
+    <row r="36" spans="1:9" ht="13" customHeight="1">
+      <c r="A36" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D36" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E36" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="F36" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F32" s="6" t="s">
+      <c r="G36" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G32" s="6" t="s">
+      <c r="H36" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H32" s="7"/>
-    </row>
-    <row r="33" spans="1:8" ht="13" customHeight="1">
-      <c r="A33" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C33" s="6" t="s">
+      <c r="I36" s="15"/>
+    </row>
+    <row r="37" spans="1:9" ht="13" customHeight="1">
+      <c r="A37" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C37" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D33" s="6" t="s">
+      <c r="D37" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E37" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="F37" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F33" s="6" t="s">
+      <c r="G37" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G33" s="6" t="s">
+      <c r="H37" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H33" s="7"/>
-    </row>
-    <row r="34" spans="1:8" ht="14">
-      <c r="A34" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C34" s="6" t="s">
+      <c r="I37" s="15"/>
+    </row>
+    <row r="38" spans="1:9" ht="14">
+      <c r="A38" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C38" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D38" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E38" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="F38" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="G38" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="G34" s="7" t="s">
+      <c r="H38" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H34" s="7"/>
-    </row>
-    <row r="35" spans="1:8" ht="13" customHeight="1">
-      <c r="A35" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C35" s="6" t="s">
+      <c r="I38" s="15"/>
+    </row>
+    <row r="39" spans="1:9" ht="13" customHeight="1">
+      <c r="A39" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C39" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D39" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E39" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="F39" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F35" s="7" t="s">
+      <c r="G39" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="G35" s="7" t="s">
+      <c r="H39" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H35" s="7"/>
-    </row>
-    <row r="36" spans="1:8" ht="13" customHeight="1">
-      <c r="A36" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C36" s="6" t="s">
+      <c r="I39" s="15"/>
+    </row>
+    <row r="40" spans="1:9" ht="13" customHeight="1">
+      <c r="A40" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D40" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E40" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="F40" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F36" s="6" t="s">
+      <c r="G40" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G36" s="6" t="s">
+      <c r="H40" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H36" s="7"/>
-    </row>
-    <row r="37" spans="1:8" ht="13" customHeight="1">
-      <c r="A37" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C37" s="6" t="s">
+      <c r="I40" s="15"/>
+    </row>
+    <row r="41" spans="1:9" ht="13" customHeight="1">
+      <c r="A41" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C41" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D37" s="6" t="s">
+      <c r="D41" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E41" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="E37" s="6" t="s">
+      <c r="F41" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F37" s="6" t="s">
+      <c r="G41" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G37" s="6" t="s">
+      <c r="H41" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H37" s="7"/>
-    </row>
-    <row r="38" spans="1:8" ht="13" customHeight="1">
-      <c r="A38" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C38" s="6" t="s">
+      <c r="I41" s="15"/>
+    </row>
+    <row r="42" spans="1:9" ht="13" customHeight="1">
+      <c r="A42" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D42" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E42" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="F42" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F38" s="6" t="s">
+      <c r="G42" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="G38" s="6" t="s">
+      <c r="H42" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H38" s="7"/>
-    </row>
-    <row r="39" spans="1:8" ht="14">
-      <c r="A39" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C39" s="7" t="s">
+      <c r="I42" s="15"/>
+    </row>
+    <row r="43" spans="1:9" ht="15">
+      <c r="A43" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C43" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D43" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E43" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="E39" s="7" t="s">
+      <c r="F43" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="F39" s="7"/>
-      <c r="G39" s="7"/>
-      <c r="H39" s="7" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="14">
-      <c r="A40" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B40" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="E40" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="G40" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="H40" s="7" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="14">
-      <c r="A41" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B41" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C41" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="E41" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="G41" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="H41" s="7" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" ht="14">
-      <c r="A42" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B42" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="D42" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="E42" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="G42" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="H42" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="14">
-      <c r="A43" s="7"/>
-      <c r="B43" s="7"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="7"/>
-      <c r="E43" s="7"/>
-      <c r="F43" s="7"/>
       <c r="G43" s="7"/>
       <c r="H43" s="7"/>
-    </row>
-    <row r="44" spans="1:8" ht="14">
-      <c r="A44" s="7"/>
-      <c r="B44" s="7"/>
-      <c r="C44" s="7"/>
-      <c r="D44" s="7"/>
-      <c r="E44" s="7"/>
-      <c r="F44" s="7"/>
-      <c r="G44" s="7"/>
-      <c r="H44" s="7"/>
-    </row>
-    <row r="45" spans="1:8" ht="14">
-      <c r="A45" s="7"/>
-      <c r="B45" s="7"/>
-      <c r="C45" s="7"/>
-      <c r="D45" s="7"/>
-      <c r="E45" s="7"/>
-      <c r="F45" s="7"/>
-      <c r="G45" s="7"/>
-      <c r="H45" s="7"/>
-    </row>
-    <row r="46" spans="1:8" ht="14">
-      <c r="A46" s="7"/>
-      <c r="B46" s="7"/>
-      <c r="C46" s="7"/>
-      <c r="D46" s="7"/>
-      <c r="E46" s="7"/>
-      <c r="F46" s="7"/>
-      <c r="G46" s="7"/>
-      <c r="H46" s="7"/>
-    </row>
-    <row r="47" spans="1:8">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="5"/>
-      <c r="D47" s="5"/>
-      <c r="E47" s="5"/>
-      <c r="F47" s="5"/>
-    </row>
-    <row r="48" spans="1:8">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="5"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
-    </row>
-    <row r="49" spans="1:6">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-    </row>
-    <row r="50" spans="1:6">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="5"/>
-      <c r="D50" s="5"/>
-      <c r="E50" s="5"/>
-      <c r="F50" s="5"/>
-    </row>
-    <row r="51" spans="1:6">
+      <c r="I43" s="15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="30">
+      <c r="A44" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I44" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="30">
+      <c r="A45" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I45" s="15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="30">
+      <c r="A46" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G46" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="H46" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="I46" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="14">
+      <c r="A47" s="7"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="15"/>
+    </row>
+    <row r="48" spans="1:9" ht="14">
+      <c r="A48" s="7"/>
+      <c r="B48" s="7"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="15"/>
+    </row>
+    <row r="49" spans="1:9" ht="14">
+      <c r="A49" s="7"/>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="15"/>
+    </row>
+    <row r="50" spans="1:9" ht="14">
+      <c r="A50" s="7"/>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="7"/>
+      <c r="I50" s="15"/>
+    </row>
+    <row r="51" spans="1:9">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="5"/>
       <c r="D51" s="5"/>
       <c r="E51" s="5"/>
       <c r="F51" s="5"/>
-    </row>
-    <row r="52" spans="1:6">
+      <c r="G51" s="5"/>
+    </row>
+    <row r="52" spans="1:9">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
       <c r="E52" s="5"/>
       <c r="F52" s="5"/>
-    </row>
-    <row r="53" spans="1:6">
+      <c r="G52" s="5"/>
+    </row>
+    <row r="53" spans="1:9">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
-    </row>
-    <row r="54" spans="1:6">
+      <c r="C53" s="5"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
+      <c r="G53" s="5"/>
+    </row>
+    <row r="54" spans="1:9">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
-    </row>
-    <row r="55" spans="1:6">
+      <c r="C54" s="5"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="5"/>
+      <c r="F54" s="5"/>
+      <c r="G54" s="5"/>
+    </row>
+    <row r="55" spans="1:9">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
-    </row>
-    <row r="56" spans="1:6">
+      <c r="C55" s="5"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
+    </row>
+    <row r="56" spans="1:9">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
-    </row>
-    <row r="57" spans="1:6">
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+    </row>
+    <row r="57" spans="1:9">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:9">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:9">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:9">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:9">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:9">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:9">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:9">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
     </row>
-    <row r="65" spans="1:7">
+    <row r="65" spans="1:4">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
     </row>
-    <row r="66" spans="1:7">
+    <row r="66" spans="1:4">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
     </row>
-    <row r="67" spans="1:7" ht="14">
+    <row r="67" spans="1:4">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
-      <c r="C67" s="2"/>
-    </row>
-    <row r="68" spans="1:7">
+    </row>
+    <row r="68" spans="1:4">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
     </row>
-    <row r="69" spans="1:7">
+    <row r="69" spans="1:4">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
     </row>
-    <row r="70" spans="1:7">
+    <row r="70" spans="1:4">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
     </row>
-    <row r="71" spans="1:7">
+    <row r="71" spans="1:4" ht="14">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
-    </row>
-    <row r="72" spans="1:7">
+      <c r="C71" s="2"/>
+      <c r="D71" s="2"/>
+    </row>
+    <row r="72" spans="1:4">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
     </row>
-    <row r="73" spans="1:7">
+    <row r="73" spans="1:4">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
     </row>
-    <row r="74" spans="1:7">
+    <row r="74" spans="1:4">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
     </row>
-    <row r="75" spans="1:7">
+    <row r="75" spans="1:4">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
     </row>
-    <row r="76" spans="1:7">
+    <row r="76" spans="1:4">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
     </row>
-    <row r="77" spans="1:7" ht="14">
+    <row r="77" spans="1:4">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
-      <c r="D77" s="2"/>
-      <c r="E77" s="2"/>
-      <c r="F77" s="2"/>
-      <c r="G77" s="2"/>
-    </row>
-    <row r="78" spans="1:7">
+    </row>
+    <row r="78" spans="1:4">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
     </row>
-    <row r="79" spans="1:7">
+    <row r="79" spans="1:4">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
     </row>
-    <row r="80" spans="1:7">
+    <row r="80" spans="1:4">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
     </row>
-    <row r="81" spans="1:7">
+    <row r="81" spans="1:8" ht="14">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
-    </row>
-    <row r="82" spans="1:7">
+      <c r="E81" s="2"/>
+      <c r="F81" s="2"/>
+      <c r="G81" s="2"/>
+      <c r="H81" s="2"/>
+    </row>
+    <row r="82" spans="1:8">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
     </row>
-    <row r="83" spans="1:7">
+    <row r="83" spans="1:8">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
     </row>
-    <row r="84" spans="1:7">
+    <row r="84" spans="1:8">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
     </row>
-    <row r="85" spans="1:7">
+    <row r="85" spans="1:8">
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
     </row>
-    <row r="86" spans="1:7">
+    <row r="86" spans="1:8">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
     </row>
-    <row r="87" spans="1:7" ht="14">
+    <row r="87" spans="1:8">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
-      <c r="D87" s="2"/>
-      <c r="E87" s="2"/>
-      <c r="F87" s="2"/>
-      <c r="G87" s="2"/>
-    </row>
-    <row r="88" spans="1:7">
+    </row>
+    <row r="88" spans="1:8">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
     </row>
-    <row r="89" spans="1:7" ht="14">
+    <row r="89" spans="1:8">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
-      <c r="C89" s="2"/>
-    </row>
-    <row r="90" spans="1:7">
+    </row>
+    <row r="90" spans="1:8">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
     </row>
-    <row r="91" spans="1:7">
+    <row r="91" spans="1:8" ht="14">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
-    </row>
-    <row r="92" spans="1:7">
+      <c r="E91" s="2"/>
+      <c r="F91" s="2"/>
+      <c r="G91" s="2"/>
+      <c r="H91" s="2"/>
+    </row>
+    <row r="92" spans="1:8">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
     </row>
-    <row r="93" spans="1:7">
+    <row r="93" spans="1:8" ht="14">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
-    </row>
-    <row r="94" spans="1:7">
+      <c r="C93" s="2"/>
+      <c r="D93" s="2"/>
+    </row>
+    <row r="94" spans="1:8">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
     </row>
-    <row r="95" spans="1:7">
+    <row r="95" spans="1:8">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
     </row>
-    <row r="96" spans="1:7" ht="14">
+    <row r="96" spans="1:8">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
-      <c r="C96" s="4"/>
-    </row>
-    <row r="97" spans="1:3" ht="14">
+    </row>
+    <row r="97" spans="1:4">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
-      <c r="C97" s="2"/>
-    </row>
-    <row r="98" spans="1:3" ht="14">
+    </row>
+    <row r="98" spans="1:4">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
-      <c r="C98" s="2"/>
-    </row>
-    <row r="99" spans="1:3">
+    </row>
+    <row r="99" spans="1:4">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
     </row>
-    <row r="100" spans="1:3">
+    <row r="100" spans="1:4" ht="14">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
-    </row>
-    <row r="101" spans="1:3">
+      <c r="C100" s="4"/>
+      <c r="D100" s="4"/>
+    </row>
+    <row r="101" spans="1:4" ht="14">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
-    </row>
-    <row r="102" spans="1:3">
+      <c r="C101" s="2"/>
+      <c r="D101" s="2"/>
+    </row>
+    <row r="102" spans="1:4" ht="14">
       <c r="A102" s="3"/>
       <c r="B102" s="3"/>
-    </row>
-    <row r="103" spans="1:3">
+      <c r="C102" s="2"/>
+      <c r="D102" s="2"/>
+    </row>
+    <row r="103" spans="1:4">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
     </row>
-    <row r="104" spans="1:3">
+    <row r="104" spans="1:4">
       <c r="A104" s="3"/>
       <c r="B104" s="3"/>
     </row>
-    <row r="105" spans="1:3">
+    <row r="105" spans="1:4">
       <c r="A105" s="3"/>
       <c r="B105" s="3"/>
     </row>
-    <row r="106" spans="1:3">
+    <row r="106" spans="1:4">
       <c r="A106" s="3"/>
       <c r="B106" s="3"/>
     </row>
-    <row r="107" spans="1:3">
+    <row r="107" spans="1:4">
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
     </row>
-    <row r="108" spans="1:3">
+    <row r="108" spans="1:4">
       <c r="A108" s="3"/>
       <c r="B108" s="3"/>
     </row>
-    <row r="109" spans="1:3">
+    <row r="109" spans="1:4">
       <c r="A109" s="3"/>
       <c r="B109" s="3"/>
     </row>
-    <row r="110" spans="1:3">
+    <row r="110" spans="1:4">
       <c r="A110" s="3"/>
       <c r="B110" s="3"/>
     </row>
-    <row r="111" spans="1:3">
+    <row r="111" spans="1:4">
       <c r="A111" s="3"/>
       <c r="B111" s="3"/>
     </row>
-    <row r="112" spans="1:3">
+    <row r="112" spans="1:4">
       <c r="A112" s="3"/>
       <c r="B112" s="3"/>
     </row>
-    <row r="113" spans="1:3">
+    <row r="113" spans="1:2">
       <c r="A113" s="3"/>
       <c r="B113" s="3"/>
     </row>
-    <row r="114" spans="1:3">
+    <row r="114" spans="1:2">
       <c r="A114" s="3"/>
       <c r="B114" s="3"/>
     </row>
-    <row r="115" spans="1:3">
+    <row r="115" spans="1:2">
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
     </row>
-    <row r="116" spans="1:3">
+    <row r="116" spans="1:2">
       <c r="A116" s="3"/>
       <c r="B116" s="3"/>
     </row>
-    <row r="117" spans="1:3">
+    <row r="117" spans="1:2">
       <c r="A117" s="3"/>
       <c r="B117" s="3"/>
     </row>
-    <row r="118" spans="1:3">
+    <row r="118" spans="1:2">
       <c r="A118" s="3"/>
       <c r="B118" s="3"/>
     </row>
-    <row r="119" spans="1:3">
+    <row r="119" spans="1:2">
       <c r="A119" s="3"/>
       <c r="B119" s="3"/>
     </row>
-    <row r="120" spans="1:3">
+    <row r="120" spans="1:2">
       <c r="A120" s="3"/>
       <c r="B120" s="3"/>
     </row>
-    <row r="121" spans="1:3">
+    <row r="121" spans="1:2">
       <c r="A121" s="3"/>
       <c r="B121" s="3"/>
     </row>
-    <row r="122" spans="1:3">
+    <row r="122" spans="1:2">
       <c r="A122" s="3"/>
       <c r="B122" s="3"/>
     </row>
-    <row r="123" spans="1:3">
+    <row r="123" spans="1:2">
       <c r="A123" s="3"/>
       <c r="B123" s="3"/>
     </row>
-    <row r="124" spans="1:3">
+    <row r="124" spans="1:2">
       <c r="A124" s="3"/>
       <c r="B124" s="3"/>
     </row>
-    <row r="125" spans="1:3">
+    <row r="125" spans="1:2">
       <c r="A125" s="3"/>
       <c r="B125" s="3"/>
     </row>
-    <row r="126" spans="1:3">
+    <row r="126" spans="1:2">
       <c r="A126" s="3"/>
       <c r="B126" s="3"/>
     </row>
-    <row r="127" spans="1:3">
+    <row r="127" spans="1:2">
       <c r="A127" s="3"/>
       <c r="B127" s="3"/>
     </row>
-    <row r="128" spans="1:3" ht="14">
+    <row r="128" spans="1:2">
       <c r="A128" s="3"/>
       <c r="B128" s="3"/>
-      <c r="C128" s="2"/>
-    </row>
-    <row r="129" spans="1:7">
+    </row>
+    <row r="129" spans="1:8">
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
     </row>
-    <row r="130" spans="1:7">
+    <row r="130" spans="1:8">
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
     </row>
-    <row r="131" spans="1:7">
+    <row r="131" spans="1:8">
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
     </row>
-    <row r="132" spans="1:7">
+    <row r="132" spans="1:8" ht="14">
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
-    </row>
-    <row r="133" spans="1:7">
+      <c r="C132" s="2"/>
+      <c r="D132" s="2"/>
+    </row>
+    <row r="133" spans="1:8">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
     </row>
-    <row r="134" spans="1:7">
+    <row r="134" spans="1:8">
       <c r="A134" s="3"/>
       <c r="B134" s="3"/>
     </row>
-    <row r="135" spans="1:7">
+    <row r="135" spans="1:8">
       <c r="A135" s="3"/>
       <c r="B135" s="3"/>
     </row>
-    <row r="136" spans="1:7" ht="14">
+    <row r="136" spans="1:8">
       <c r="A136" s="3"/>
       <c r="B136" s="3"/>
-      <c r="D136" s="4"/>
-      <c r="E136" s="4"/>
-      <c r="F136" s="4"/>
-      <c r="G136" s="4"/>
-    </row>
-    <row r="137" spans="1:7" ht="14">
+    </row>
+    <row r="137" spans="1:8">
       <c r="A137" s="3"/>
       <c r="B137" s="3"/>
-      <c r="D137" s="2"/>
-      <c r="E137" s="2"/>
-      <c r="F137" s="2"/>
-      <c r="G137" s="2"/>
-    </row>
-    <row r="138" spans="1:7" ht="14">
+    </row>
+    <row r="138" spans="1:8">
       <c r="A138" s="3"/>
       <c r="B138" s="3"/>
-      <c r="C138" s="2"/>
-    </row>
-    <row r="139" spans="1:7">
+    </row>
+    <row r="139" spans="1:8">
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
     </row>
-    <row r="140" spans="1:7">
+    <row r="140" spans="1:8" ht="14">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
-    </row>
-    <row r="141" spans="1:7">
+      <c r="E140" s="4"/>
+      <c r="F140" s="4"/>
+      <c r="G140" s="4"/>
+      <c r="H140" s="4"/>
+    </row>
+    <row r="141" spans="1:8" ht="14">
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
-    </row>
-    <row r="142" spans="1:7">
+      <c r="E141" s="2"/>
+      <c r="F141" s="2"/>
+      <c r="G141" s="2"/>
+      <c r="H141" s="2"/>
+    </row>
+    <row r="142" spans="1:8" ht="14">
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
-    </row>
-    <row r="143" spans="1:7">
+      <c r="C142" s="2"/>
+      <c r="D142" s="2"/>
+    </row>
+    <row r="143" spans="1:8">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
     </row>
-    <row r="144" spans="1:7">
+    <row r="144" spans="1:8">
       <c r="A144" s="3"/>
       <c r="B144" s="3"/>
     </row>
-    <row r="145" spans="1:7">
+    <row r="145" spans="1:8">
       <c r="A145" s="3"/>
       <c r="B145" s="3"/>
     </row>
-    <row r="146" spans="1:7">
+    <row r="146" spans="1:8">
       <c r="A146" s="3"/>
       <c r="B146" s="3"/>
     </row>
-    <row r="147" spans="1:7">
+    <row r="147" spans="1:8">
       <c r="A147" s="3"/>
       <c r="B147" s="3"/>
     </row>
-    <row r="148" spans="1:7" ht="14">
+    <row r="148" spans="1:8">
       <c r="A148" s="3"/>
       <c r="B148" s="3"/>
-      <c r="D148" s="2"/>
-      <c r="E148" s="2"/>
-      <c r="F148" s="2"/>
-      <c r="G148" s="2"/>
-    </row>
-    <row r="149" spans="1:7">
+    </row>
+    <row r="149" spans="1:8">
       <c r="A149" s="3"/>
       <c r="B149" s="3"/>
     </row>
-    <row r="150" spans="1:7">
+    <row r="150" spans="1:8">
       <c r="A150" s="3"/>
       <c r="B150" s="3"/>
     </row>
-    <row r="151" spans="1:7" ht="14">
+    <row r="151" spans="1:8">
       <c r="A151" s="3"/>
       <c r="B151" s="3"/>
-      <c r="D151" s="2"/>
-      <c r="E151" s="2"/>
-      <c r="F151" s="2"/>
-      <c r="G151" s="2"/>
-    </row>
-    <row r="152" spans="1:7">
+    </row>
+    <row r="152" spans="1:8" ht="14">
       <c r="A152" s="3"/>
       <c r="B152" s="3"/>
-    </row>
-    <row r="153" spans="1:7">
+      <c r="E152" s="2"/>
+      <c r="F152" s="2"/>
+      <c r="G152" s="2"/>
+      <c r="H152" s="2"/>
+    </row>
+    <row r="153" spans="1:8">
       <c r="A153" s="3"/>
       <c r="B153" s="3"/>
     </row>
-    <row r="154" spans="1:7">
+    <row r="154" spans="1:8">
       <c r="A154" s="3"/>
       <c r="B154" s="3"/>
     </row>
-    <row r="155" spans="1:7">
+    <row r="155" spans="1:8" ht="14">
       <c r="A155" s="3"/>
       <c r="B155" s="3"/>
-    </row>
-    <row r="156" spans="1:7">
+      <c r="E155" s="2"/>
+      <c r="F155" s="2"/>
+      <c r="G155" s="2"/>
+      <c r="H155" s="2"/>
+    </row>
+    <row r="156" spans="1:8">
       <c r="A156" s="3"/>
       <c r="B156" s="3"/>
     </row>
-    <row r="157" spans="1:7">
+    <row r="157" spans="1:8">
       <c r="A157" s="3"/>
       <c r="B157" s="3"/>
     </row>
-    <row r="158" spans="1:7">
+    <row r="158" spans="1:8">
       <c r="A158" s="3"/>
       <c r="B158" s="3"/>
     </row>
-    <row r="159" spans="1:7">
+    <row r="159" spans="1:8">
       <c r="A159" s="3"/>
       <c r="B159" s="3"/>
     </row>
-    <row r="160" spans="1:7">
+    <row r="160" spans="1:8">
       <c r="A160" s="3"/>
       <c r="B160" s="3"/>
     </row>
@@ -2458,751 +2730,966 @@
       <c r="A176" s="3"/>
       <c r="B176" s="3"/>
     </row>
-    <row r="177" spans="1:3">
+    <row r="177" spans="1:4">
       <c r="A177" s="3"/>
       <c r="B177" s="3"/>
     </row>
-    <row r="178" spans="1:3">
+    <row r="178" spans="1:4">
       <c r="A178" s="3"/>
       <c r="B178" s="3"/>
     </row>
-    <row r="179" spans="1:3">
+    <row r="179" spans="1:4">
       <c r="A179" s="3"/>
       <c r="B179" s="3"/>
     </row>
-    <row r="180" spans="1:3">
+    <row r="180" spans="1:4">
       <c r="A180" s="3"/>
       <c r="B180" s="3"/>
     </row>
-    <row r="181" spans="1:3">
+    <row r="181" spans="1:4">
       <c r="A181" s="3"/>
       <c r="B181" s="3"/>
     </row>
-    <row r="182" spans="1:3">
+    <row r="182" spans="1:4">
       <c r="A182" s="3"/>
       <c r="B182" s="3"/>
     </row>
-    <row r="183" spans="1:3">
+    <row r="183" spans="1:4">
       <c r="A183" s="3"/>
       <c r="B183" s="3"/>
     </row>
-    <row r="184" spans="1:3">
+    <row r="184" spans="1:4">
       <c r="A184" s="3"/>
       <c r="B184" s="3"/>
     </row>
-    <row r="185" spans="1:3">
+    <row r="185" spans="1:4">
       <c r="A185" s="3"/>
       <c r="B185" s="3"/>
     </row>
-    <row r="186" spans="1:3">
+    <row r="186" spans="1:4">
       <c r="A186" s="3"/>
       <c r="B186" s="3"/>
     </row>
-    <row r="187" spans="1:3" ht="14">
+    <row r="187" spans="1:4">
       <c r="A187" s="3"/>
       <c r="B187" s="3"/>
-      <c r="C187" s="4"/>
-    </row>
-    <row r="188" spans="1:3" ht="14">
+    </row>
+    <row r="188" spans="1:4">
       <c r="A188" s="3"/>
       <c r="B188" s="3"/>
-      <c r="C188" s="2"/>
-    </row>
-    <row r="189" spans="1:3">
+    </row>
+    <row r="189" spans="1:4">
       <c r="A189" s="3"/>
       <c r="B189" s="3"/>
     </row>
-    <row r="190" spans="1:3">
+    <row r="190" spans="1:4">
       <c r="A190" s="3"/>
       <c r="B190" s="3"/>
     </row>
-    <row r="191" spans="1:3">
+    <row r="191" spans="1:4" ht="14">
       <c r="A191" s="3"/>
       <c r="B191" s="3"/>
-    </row>
-    <row r="192" spans="1:3">
+      <c r="C191" s="4"/>
+      <c r="D191" s="4"/>
+    </row>
+    <row r="192" spans="1:4" ht="14">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
-    </row>
-    <row r="193" spans="1:3">
+      <c r="C192" s="2"/>
+      <c r="D192" s="2"/>
+    </row>
+    <row r="193" spans="1:4">
       <c r="A193" s="3"/>
       <c r="B193" s="3"/>
     </row>
-    <row r="194" spans="1:3">
+    <row r="194" spans="1:4">
       <c r="A194" s="3"/>
       <c r="B194" s="3"/>
     </row>
-    <row r="195" spans="1:3">
+    <row r="195" spans="1:4">
       <c r="A195" s="3"/>
       <c r="B195" s="3"/>
     </row>
-    <row r="196" spans="1:3">
+    <row r="196" spans="1:4">
       <c r="A196" s="3"/>
       <c r="B196" s="3"/>
     </row>
-    <row r="197" spans="1:3">
+    <row r="197" spans="1:4">
       <c r="A197" s="3"/>
       <c r="B197" s="3"/>
     </row>
-    <row r="198" spans="1:3">
+    <row r="198" spans="1:4">
       <c r="A198" s="3"/>
       <c r="B198" s="3"/>
     </row>
-    <row r="199" spans="1:3" ht="14">
+    <row r="199" spans="1:4">
       <c r="A199" s="3"/>
       <c r="B199" s="3"/>
-      <c r="C199" s="2"/>
-    </row>
-    <row r="200" spans="1:3">
+    </row>
+    <row r="200" spans="1:4">
       <c r="A200" s="3"/>
       <c r="B200" s="3"/>
     </row>
-    <row r="201" spans="1:3">
+    <row r="201" spans="1:4">
       <c r="A201" s="3"/>
       <c r="B201" s="3"/>
     </row>
-    <row r="202" spans="1:3" ht="14">
+    <row r="202" spans="1:4">
       <c r="A202" s="3"/>
       <c r="B202" s="3"/>
-      <c r="C202" s="2"/>
-    </row>
-    <row r="203" spans="1:3">
+    </row>
+    <row r="203" spans="1:4" ht="14">
       <c r="A203" s="3"/>
       <c r="B203" s="3"/>
-    </row>
-    <row r="204" spans="1:3">
+      <c r="C203" s="2"/>
+      <c r="D203" s="2"/>
+    </row>
+    <row r="204" spans="1:4">
       <c r="A204" s="3"/>
       <c r="B204" s="3"/>
     </row>
-    <row r="205" spans="1:3">
+    <row r="205" spans="1:4">
       <c r="A205" s="3"/>
       <c r="B205" s="3"/>
     </row>
-    <row r="206" spans="1:3">
+    <row r="206" spans="1:4" ht="14">
       <c r="A206" s="3"/>
       <c r="B206" s="3"/>
-    </row>
-    <row r="207" spans="1:3">
+      <c r="C206" s="2"/>
+      <c r="D206" s="2"/>
+    </row>
+    <row r="207" spans="1:4">
       <c r="A207" s="3"/>
       <c r="B207" s="3"/>
     </row>
-    <row r="208" spans="1:3">
+    <row r="208" spans="1:4">
       <c r="A208" s="3"/>
       <c r="B208" s="3"/>
     </row>
-    <row r="209" spans="1:3">
+    <row r="209" spans="1:4">
       <c r="A209" s="3"/>
       <c r="B209" s="3"/>
     </row>
-    <row r="210" spans="1:3">
+    <row r="210" spans="1:4">
       <c r="A210" s="3"/>
       <c r="B210" s="3"/>
     </row>
-    <row r="211" spans="1:3">
+    <row r="211" spans="1:4">
       <c r="A211" s="3"/>
       <c r="B211" s="3"/>
     </row>
-    <row r="212" spans="1:3">
+    <row r="212" spans="1:4">
       <c r="A212" s="3"/>
       <c r="B212" s="3"/>
-      <c r="C212" s="3"/>
-    </row>
-    <row r="213" spans="1:3">
+    </row>
+    <row r="213" spans="1:4">
       <c r="A213" s="3"/>
       <c r="B213" s="3"/>
-      <c r="C213" s="3"/>
-    </row>
-    <row r="214" spans="1:3">
+    </row>
+    <row r="214" spans="1:4">
       <c r="A214" s="3"/>
       <c r="B214" s="3"/>
-      <c r="C214" s="3"/>
-    </row>
-    <row r="215" spans="1:3">
+    </row>
+    <row r="215" spans="1:4">
       <c r="A215" s="3"/>
       <c r="B215" s="3"/>
-      <c r="C215" s="3"/>
-    </row>
-    <row r="216" spans="1:3">
+    </row>
+    <row r="216" spans="1:4">
       <c r="A216" s="3"/>
       <c r="B216" s="3"/>
       <c r="C216" s="3"/>
-    </row>
-    <row r="217" spans="1:3">
+      <c r="D216" s="3"/>
+    </row>
+    <row r="217" spans="1:4">
       <c r="A217" s="3"/>
       <c r="B217" s="3"/>
       <c r="C217" s="3"/>
-    </row>
-    <row r="218" spans="1:3">
+      <c r="D217" s="3"/>
+    </row>
+    <row r="218" spans="1:4">
+      <c r="A218" s="3"/>
+      <c r="B218" s="3"/>
       <c r="C218" s="3"/>
-    </row>
-    <row r="219" spans="1:3">
+      <c r="D218" s="3"/>
+    </row>
+    <row r="219" spans="1:4">
+      <c r="A219" s="3"/>
+      <c r="B219" s="3"/>
       <c r="C219" s="3"/>
-    </row>
-    <row r="220" spans="1:3">
+      <c r="D219" s="3"/>
+    </row>
+    <row r="220" spans="1:4">
+      <c r="A220" s="3"/>
+      <c r="B220" s="3"/>
       <c r="C220" s="3"/>
-    </row>
-    <row r="221" spans="1:3">
+      <c r="D220" s="3"/>
+    </row>
+    <row r="221" spans="1:4">
+      <c r="A221" s="3"/>
+      <c r="B221" s="3"/>
       <c r="C221" s="3"/>
-    </row>
-    <row r="222" spans="1:3">
+      <c r="D221" s="3"/>
+    </row>
+    <row r="222" spans="1:4">
       <c r="C222" s="3"/>
-    </row>
-    <row r="223" spans="1:3">
+      <c r="D222" s="3"/>
+    </row>
+    <row r="223" spans="1:4">
       <c r="C223" s="3"/>
-    </row>
-    <row r="224" spans="1:3">
+      <c r="D223" s="3"/>
+    </row>
+    <row r="224" spans="1:4">
       <c r="C224" s="3"/>
-    </row>
-    <row r="225" spans="3:3">
+      <c r="D224" s="3"/>
+    </row>
+    <row r="225" spans="3:4">
       <c r="C225" s="3"/>
-    </row>
-    <row r="226" spans="3:3">
+      <c r="D225" s="3"/>
+    </row>
+    <row r="226" spans="3:4">
       <c r="C226" s="3"/>
-    </row>
-    <row r="227" spans="3:3">
+      <c r="D226" s="3"/>
+    </row>
+    <row r="227" spans="3:4">
       <c r="C227" s="3"/>
-    </row>
-    <row r="228" spans="3:3">
+      <c r="D227" s="3"/>
+    </row>
+    <row r="228" spans="3:4">
       <c r="C228" s="3"/>
-    </row>
-    <row r="229" spans="3:3">
+      <c r="D228" s="3"/>
+    </row>
+    <row r="229" spans="3:4">
       <c r="C229" s="3"/>
-    </row>
-    <row r="230" spans="3:3">
+      <c r="D229" s="3"/>
+    </row>
+    <row r="230" spans="3:4">
       <c r="C230" s="3"/>
-    </row>
-    <row r="231" spans="3:3">
+      <c r="D230" s="3"/>
+    </row>
+    <row r="231" spans="3:4">
       <c r="C231" s="3"/>
-    </row>
-    <row r="232" spans="3:3">
+      <c r="D231" s="3"/>
+    </row>
+    <row r="232" spans="3:4">
       <c r="C232" s="3"/>
-    </row>
-    <row r="233" spans="3:3">
+      <c r="D232" s="3"/>
+    </row>
+    <row r="233" spans="3:4">
       <c r="C233" s="3"/>
-    </row>
-    <row r="234" spans="3:3">
+      <c r="D233" s="3"/>
+    </row>
+    <row r="234" spans="3:4">
       <c r="C234" s="3"/>
-    </row>
-    <row r="235" spans="3:3">
+      <c r="D234" s="3"/>
+    </row>
+    <row r="235" spans="3:4">
       <c r="C235" s="3"/>
-    </row>
-    <row r="236" spans="3:3">
+      <c r="D235" s="3"/>
+    </row>
+    <row r="236" spans="3:4">
       <c r="C236" s="3"/>
-    </row>
-    <row r="237" spans="3:3">
+      <c r="D236" s="3"/>
+    </row>
+    <row r="237" spans="3:4">
       <c r="C237" s="3"/>
-    </row>
-    <row r="238" spans="3:3">
+      <c r="D237" s="3"/>
+    </row>
+    <row r="238" spans="3:4">
       <c r="C238" s="3"/>
-    </row>
-    <row r="239" spans="3:3">
+      <c r="D238" s="3"/>
+    </row>
+    <row r="239" spans="3:4">
       <c r="C239" s="3"/>
-    </row>
-    <row r="240" spans="3:3">
+      <c r="D239" s="3"/>
+    </row>
+    <row r="240" spans="3:4">
       <c r="C240" s="3"/>
-    </row>
-    <row r="241" spans="3:3">
+      <c r="D240" s="3"/>
+    </row>
+    <row r="241" spans="3:4">
       <c r="C241" s="3"/>
-    </row>
-    <row r="242" spans="3:3">
+      <c r="D241" s="3"/>
+    </row>
+    <row r="242" spans="3:4">
       <c r="C242" s="3"/>
-    </row>
-    <row r="243" spans="3:3">
+      <c r="D242" s="3"/>
+    </row>
+    <row r="243" spans="3:4">
       <c r="C243" s="3"/>
-    </row>
-    <row r="244" spans="3:3">
+      <c r="D243" s="3"/>
+    </row>
+    <row r="244" spans="3:4">
       <c r="C244" s="3"/>
-    </row>
-    <row r="245" spans="3:3">
+      <c r="D244" s="3"/>
+    </row>
+    <row r="245" spans="3:4">
       <c r="C245" s="3"/>
-    </row>
-    <row r="246" spans="3:3">
+      <c r="D245" s="3"/>
+    </row>
+    <row r="246" spans="3:4">
       <c r="C246" s="3"/>
-    </row>
-    <row r="247" spans="3:3">
+      <c r="D246" s="3"/>
+    </row>
+    <row r="247" spans="3:4">
       <c r="C247" s="3"/>
-    </row>
-    <row r="248" spans="3:3">
+      <c r="D247" s="3"/>
+    </row>
+    <row r="248" spans="3:4">
       <c r="C248" s="3"/>
-    </row>
-    <row r="249" spans="3:3">
+      <c r="D248" s="3"/>
+    </row>
+    <row r="249" spans="3:4">
       <c r="C249" s="3"/>
-    </row>
-    <row r="250" spans="3:3">
+      <c r="D249" s="3"/>
+    </row>
+    <row r="250" spans="3:4">
       <c r="C250" s="3"/>
-    </row>
-    <row r="251" spans="3:3">
+      <c r="D250" s="3"/>
+    </row>
+    <row r="251" spans="3:4">
       <c r="C251" s="3"/>
-    </row>
-    <row r="252" spans="3:3">
+      <c r="D251" s="3"/>
+    </row>
+    <row r="252" spans="3:4">
       <c r="C252" s="3"/>
-    </row>
-    <row r="253" spans="3:3">
+      <c r="D252" s="3"/>
+    </row>
+    <row r="253" spans="3:4">
       <c r="C253" s="3"/>
-    </row>
-    <row r="254" spans="3:3">
+      <c r="D253" s="3"/>
+    </row>
+    <row r="254" spans="3:4">
       <c r="C254" s="3"/>
-    </row>
-    <row r="255" spans="3:3">
+      <c r="D254" s="3"/>
+    </row>
+    <row r="255" spans="3:4">
       <c r="C255" s="3"/>
-    </row>
-    <row r="256" spans="3:3">
+      <c r="D255" s="3"/>
+    </row>
+    <row r="256" spans="3:4">
       <c r="C256" s="3"/>
-    </row>
-    <row r="257" spans="3:3">
+      <c r="D256" s="3"/>
+    </row>
+    <row r="257" spans="3:4">
       <c r="C257" s="3"/>
-    </row>
-    <row r="258" spans="3:3">
+      <c r="D257" s="3"/>
+    </row>
+    <row r="258" spans="3:4">
       <c r="C258" s="3"/>
-    </row>
-    <row r="259" spans="3:3">
+      <c r="D258" s="3"/>
+    </row>
+    <row r="259" spans="3:4">
       <c r="C259" s="3"/>
-    </row>
-    <row r="260" spans="3:3">
+      <c r="D259" s="3"/>
+    </row>
+    <row r="260" spans="3:4">
       <c r="C260" s="3"/>
-    </row>
-    <row r="261" spans="3:3">
+      <c r="D260" s="3"/>
+    </row>
+    <row r="261" spans="3:4">
       <c r="C261" s="3"/>
-    </row>
-    <row r="262" spans="3:3">
+      <c r="D261" s="3"/>
+    </row>
+    <row r="262" spans="3:4">
       <c r="C262" s="3"/>
-    </row>
-    <row r="263" spans="3:3">
+      <c r="D262" s="3"/>
+    </row>
+    <row r="263" spans="3:4">
       <c r="C263" s="3"/>
-    </row>
-    <row r="264" spans="3:3">
+      <c r="D263" s="3"/>
+    </row>
+    <row r="264" spans="3:4">
       <c r="C264" s="3"/>
-    </row>
-    <row r="265" spans="3:3">
+      <c r="D264" s="3"/>
+    </row>
+    <row r="265" spans="3:4">
       <c r="C265" s="3"/>
-    </row>
-    <row r="266" spans="3:3">
+      <c r="D265" s="3"/>
+    </row>
+    <row r="266" spans="3:4">
       <c r="C266" s="3"/>
-    </row>
-    <row r="267" spans="3:3">
+      <c r="D266" s="3"/>
+    </row>
+    <row r="267" spans="3:4">
       <c r="C267" s="3"/>
-    </row>
-    <row r="268" spans="3:3">
+      <c r="D267" s="3"/>
+    </row>
+    <row r="268" spans="3:4">
       <c r="C268" s="3"/>
-    </row>
-    <row r="269" spans="3:3">
+      <c r="D268" s="3"/>
+    </row>
+    <row r="269" spans="3:4">
       <c r="C269" s="3"/>
-    </row>
-    <row r="270" spans="3:3">
+      <c r="D269" s="3"/>
+    </row>
+    <row r="270" spans="3:4">
       <c r="C270" s="3"/>
-    </row>
-    <row r="271" spans="3:3">
+      <c r="D270" s="3"/>
+    </row>
+    <row r="271" spans="3:4">
       <c r="C271" s="3"/>
-    </row>
-    <row r="272" spans="3:3">
+      <c r="D271" s="3"/>
+    </row>
+    <row r="272" spans="3:4">
       <c r="C272" s="3"/>
-    </row>
-    <row r="273" spans="3:3">
+      <c r="D272" s="3"/>
+    </row>
+    <row r="273" spans="3:4">
       <c r="C273" s="3"/>
-    </row>
-    <row r="274" spans="3:3">
+      <c r="D273" s="3"/>
+    </row>
+    <row r="274" spans="3:4">
       <c r="C274" s="3"/>
-    </row>
-    <row r="275" spans="3:3">
+      <c r="D274" s="3"/>
+    </row>
+    <row r="275" spans="3:4">
       <c r="C275" s="3"/>
-    </row>
-    <row r="276" spans="3:3">
+      <c r="D275" s="3"/>
+    </row>
+    <row r="276" spans="3:4">
       <c r="C276" s="3"/>
-    </row>
-    <row r="277" spans="3:3">
+      <c r="D276" s="3"/>
+    </row>
+    <row r="277" spans="3:4">
       <c r="C277" s="3"/>
-    </row>
-    <row r="278" spans="3:3">
+      <c r="D277" s="3"/>
+    </row>
+    <row r="278" spans="3:4">
       <c r="C278" s="3"/>
-    </row>
-    <row r="279" spans="3:3">
+      <c r="D278" s="3"/>
+    </row>
+    <row r="279" spans="3:4">
       <c r="C279" s="3"/>
-    </row>
-    <row r="280" spans="3:3">
+      <c r="D279" s="3"/>
+    </row>
+    <row r="280" spans="3:4">
       <c r="C280" s="3"/>
-    </row>
-    <row r="281" spans="3:3">
+      <c r="D280" s="3"/>
+    </row>
+    <row r="281" spans="3:4">
       <c r="C281" s="3"/>
-    </row>
-    <row r="282" spans="3:3">
+      <c r="D281" s="3"/>
+    </row>
+    <row r="282" spans="3:4">
       <c r="C282" s="3"/>
-    </row>
-    <row r="283" spans="3:3">
+      <c r="D282" s="3"/>
+    </row>
+    <row r="283" spans="3:4">
       <c r="C283" s="3"/>
-    </row>
-    <row r="284" spans="3:3">
+      <c r="D283" s="3"/>
+    </row>
+    <row r="284" spans="3:4">
       <c r="C284" s="3"/>
-    </row>
-    <row r="285" spans="3:3">
+      <c r="D284" s="3"/>
+    </row>
+    <row r="285" spans="3:4">
       <c r="C285" s="3"/>
-    </row>
-    <row r="286" spans="3:3">
+      <c r="D285" s="3"/>
+    </row>
+    <row r="286" spans="3:4">
       <c r="C286" s="3"/>
-    </row>
-    <row r="287" spans="3:3">
+      <c r="D286" s="3"/>
+    </row>
+    <row r="287" spans="3:4">
       <c r="C287" s="3"/>
-    </row>
-    <row r="288" spans="3:3">
+      <c r="D287" s="3"/>
+    </row>
+    <row r="288" spans="3:4">
       <c r="C288" s="3"/>
-    </row>
-    <row r="289" spans="3:3">
+      <c r="D288" s="3"/>
+    </row>
+    <row r="289" spans="3:4">
       <c r="C289" s="3"/>
-    </row>
-    <row r="290" spans="3:3">
+      <c r="D289" s="3"/>
+    </row>
+    <row r="290" spans="3:4">
       <c r="C290" s="3"/>
-    </row>
-    <row r="291" spans="3:3">
+      <c r="D290" s="3"/>
+    </row>
+    <row r="291" spans="3:4">
       <c r="C291" s="3"/>
-    </row>
-    <row r="292" spans="3:3">
+      <c r="D291" s="3"/>
+    </row>
+    <row r="292" spans="3:4">
       <c r="C292" s="3"/>
-    </row>
-    <row r="293" spans="3:3">
+      <c r="D292" s="3"/>
+    </row>
+    <row r="293" spans="3:4">
       <c r="C293" s="3"/>
-    </row>
-    <row r="294" spans="3:3">
+      <c r="D293" s="3"/>
+    </row>
+    <row r="294" spans="3:4">
       <c r="C294" s="3"/>
-    </row>
-    <row r="295" spans="3:3">
+      <c r="D294" s="3"/>
+    </row>
+    <row r="295" spans="3:4">
       <c r="C295" s="3"/>
-    </row>
-    <row r="296" spans="3:3">
+      <c r="D295" s="3"/>
+    </row>
+    <row r="296" spans="3:4">
       <c r="C296" s="3"/>
-    </row>
-    <row r="297" spans="3:3">
+      <c r="D296" s="3"/>
+    </row>
+    <row r="297" spans="3:4">
       <c r="C297" s="3"/>
-    </row>
-    <row r="298" spans="3:3">
+      <c r="D297" s="3"/>
+    </row>
+    <row r="298" spans="3:4">
       <c r="C298" s="3"/>
-    </row>
-    <row r="299" spans="3:3">
+      <c r="D298" s="3"/>
+    </row>
+    <row r="299" spans="3:4">
       <c r="C299" s="3"/>
-    </row>
-    <row r="300" spans="3:3">
+      <c r="D299" s="3"/>
+    </row>
+    <row r="300" spans="3:4">
       <c r="C300" s="3"/>
-    </row>
-    <row r="301" spans="3:3">
+      <c r="D300" s="3"/>
+    </row>
+    <row r="301" spans="3:4">
       <c r="C301" s="3"/>
-    </row>
-    <row r="302" spans="3:3">
+      <c r="D301" s="3"/>
+    </row>
+    <row r="302" spans="3:4">
       <c r="C302" s="3"/>
-    </row>
-    <row r="303" spans="3:3">
+      <c r="D302" s="3"/>
+    </row>
+    <row r="303" spans="3:4">
       <c r="C303" s="3"/>
-    </row>
-    <row r="304" spans="3:3">
+      <c r="D303" s="3"/>
+    </row>
+    <row r="304" spans="3:4">
       <c r="C304" s="3"/>
-    </row>
-    <row r="305" spans="3:3">
+      <c r="D304" s="3"/>
+    </row>
+    <row r="305" spans="3:4">
       <c r="C305" s="3"/>
-    </row>
-    <row r="306" spans="3:3">
+      <c r="D305" s="3"/>
+    </row>
+    <row r="306" spans="3:4">
       <c r="C306" s="3"/>
-    </row>
-    <row r="307" spans="3:3">
+      <c r="D306" s="3"/>
+    </row>
+    <row r="307" spans="3:4">
       <c r="C307" s="3"/>
-    </row>
-    <row r="308" spans="3:3">
+      <c r="D307" s="3"/>
+    </row>
+    <row r="308" spans="3:4">
       <c r="C308" s="3"/>
-    </row>
-    <row r="309" spans="3:3">
+      <c r="D308" s="3"/>
+    </row>
+    <row r="309" spans="3:4">
       <c r="C309" s="3"/>
-    </row>
-    <row r="310" spans="3:3">
+      <c r="D309" s="3"/>
+    </row>
+    <row r="310" spans="3:4">
       <c r="C310" s="3"/>
-    </row>
-    <row r="311" spans="3:3">
+      <c r="D310" s="3"/>
+    </row>
+    <row r="311" spans="3:4">
       <c r="C311" s="3"/>
-    </row>
-    <row r="312" spans="3:3">
+      <c r="D311" s="3"/>
+    </row>
+    <row r="312" spans="3:4">
       <c r="C312" s="3"/>
-    </row>
-    <row r="313" spans="3:3">
+      <c r="D312" s="3"/>
+    </row>
+    <row r="313" spans="3:4">
       <c r="C313" s="3"/>
-    </row>
-    <row r="314" spans="3:3">
+      <c r="D313" s="3"/>
+    </row>
+    <row r="314" spans="3:4">
       <c r="C314" s="3"/>
-    </row>
-    <row r="315" spans="3:3">
+      <c r="D314" s="3"/>
+    </row>
+    <row r="315" spans="3:4">
       <c r="C315" s="3"/>
-    </row>
-    <row r="316" spans="3:3">
+      <c r="D315" s="3"/>
+    </row>
+    <row r="316" spans="3:4">
       <c r="C316" s="3"/>
-    </row>
-    <row r="317" spans="3:3">
+      <c r="D316" s="3"/>
+    </row>
+    <row r="317" spans="3:4">
       <c r="C317" s="3"/>
-    </row>
-    <row r="318" spans="3:3">
+      <c r="D317" s="3"/>
+    </row>
+    <row r="318" spans="3:4">
       <c r="C318" s="3"/>
-    </row>
-    <row r="319" spans="3:3">
+      <c r="D318" s="3"/>
+    </row>
+    <row r="319" spans="3:4">
       <c r="C319" s="3"/>
-    </row>
-    <row r="320" spans="3:3">
+      <c r="D319" s="3"/>
+    </row>
+    <row r="320" spans="3:4">
       <c r="C320" s="3"/>
-    </row>
-    <row r="321" spans="3:3">
+      <c r="D320" s="3"/>
+    </row>
+    <row r="321" spans="3:4">
       <c r="C321" s="3"/>
-    </row>
-    <row r="322" spans="3:3">
+      <c r="D321" s="3"/>
+    </row>
+    <row r="322" spans="3:4">
       <c r="C322" s="3"/>
-    </row>
-    <row r="323" spans="3:3">
+      <c r="D322" s="3"/>
+    </row>
+    <row r="323" spans="3:4">
       <c r="C323" s="3"/>
-    </row>
-    <row r="324" spans="3:3">
+      <c r="D323" s="3"/>
+    </row>
+    <row r="324" spans="3:4">
       <c r="C324" s="3"/>
-    </row>
-    <row r="325" spans="3:3">
+      <c r="D324" s="3"/>
+    </row>
+    <row r="325" spans="3:4">
       <c r="C325" s="3"/>
-    </row>
-    <row r="326" spans="3:3">
+      <c r="D325" s="3"/>
+    </row>
+    <row r="326" spans="3:4">
       <c r="C326" s="3"/>
-    </row>
-    <row r="327" spans="3:3">
+      <c r="D326" s="3"/>
+    </row>
+    <row r="327" spans="3:4">
       <c r="C327" s="3"/>
-    </row>
-    <row r="328" spans="3:3">
+      <c r="D327" s="3"/>
+    </row>
+    <row r="328" spans="3:4">
       <c r="C328" s="3"/>
-    </row>
-    <row r="329" spans="3:3">
+      <c r="D328" s="3"/>
+    </row>
+    <row r="329" spans="3:4">
       <c r="C329" s="3"/>
-    </row>
-    <row r="330" spans="3:3">
+      <c r="D329" s="3"/>
+    </row>
+    <row r="330" spans="3:4">
       <c r="C330" s="3"/>
-    </row>
-    <row r="331" spans="3:3">
+      <c r="D330" s="3"/>
+    </row>
+    <row r="331" spans="3:4">
       <c r="C331" s="3"/>
-    </row>
-    <row r="332" spans="3:3">
+      <c r="D331" s="3"/>
+    </row>
+    <row r="332" spans="3:4">
       <c r="C332" s="3"/>
-    </row>
-    <row r="333" spans="3:3">
+      <c r="D332" s="3"/>
+    </row>
+    <row r="333" spans="3:4">
       <c r="C333" s="3"/>
-    </row>
-    <row r="334" spans="3:3">
+      <c r="D333" s="3"/>
+    </row>
+    <row r="334" spans="3:4">
       <c r="C334" s="3"/>
-    </row>
-    <row r="335" spans="3:3">
+      <c r="D334" s="3"/>
+    </row>
+    <row r="335" spans="3:4">
       <c r="C335" s="3"/>
-    </row>
-    <row r="336" spans="3:3">
+      <c r="D335" s="3"/>
+    </row>
+    <row r="336" spans="3:4">
       <c r="C336" s="3"/>
-    </row>
-    <row r="337" spans="3:3">
+      <c r="D336" s="3"/>
+    </row>
+    <row r="337" spans="3:4">
       <c r="C337" s="3"/>
-    </row>
-    <row r="338" spans="3:3">
+      <c r="D337" s="3"/>
+    </row>
+    <row r="338" spans="3:4">
       <c r="C338" s="3"/>
-    </row>
-    <row r="339" spans="3:3">
+      <c r="D338" s="3"/>
+    </row>
+    <row r="339" spans="3:4">
       <c r="C339" s="3"/>
-    </row>
-    <row r="340" spans="3:3">
+      <c r="D339" s="3"/>
+    </row>
+    <row r="340" spans="3:4">
       <c r="C340" s="3"/>
-    </row>
-    <row r="341" spans="3:3">
+      <c r="D340" s="3"/>
+    </row>
+    <row r="341" spans="3:4">
       <c r="C341" s="3"/>
-    </row>
-    <row r="342" spans="3:3">
+      <c r="D341" s="3"/>
+    </row>
+    <row r="342" spans="3:4">
       <c r="C342" s="3"/>
-    </row>
-    <row r="343" spans="3:3">
+      <c r="D342" s="3"/>
+    </row>
+    <row r="343" spans="3:4">
       <c r="C343" s="3"/>
-    </row>
-    <row r="344" spans="3:3">
+      <c r="D343" s="3"/>
+    </row>
+    <row r="344" spans="3:4">
       <c r="C344" s="3"/>
-    </row>
-    <row r="345" spans="3:3">
+      <c r="D344" s="3"/>
+    </row>
+    <row r="345" spans="3:4">
       <c r="C345" s="3"/>
-    </row>
-    <row r="346" spans="3:3">
+      <c r="D345" s="3"/>
+    </row>
+    <row r="346" spans="3:4">
       <c r="C346" s="3"/>
-    </row>
-    <row r="347" spans="3:3">
+      <c r="D346" s="3"/>
+    </row>
+    <row r="347" spans="3:4">
       <c r="C347" s="3"/>
-    </row>
-    <row r="348" spans="3:3">
+      <c r="D347" s="3"/>
+    </row>
+    <row r="348" spans="3:4">
       <c r="C348" s="3"/>
-    </row>
-    <row r="349" spans="3:3">
+      <c r="D348" s="3"/>
+    </row>
+    <row r="349" spans="3:4">
       <c r="C349" s="3"/>
-    </row>
-    <row r="350" spans="3:3">
+      <c r="D349" s="3"/>
+    </row>
+    <row r="350" spans="3:4">
       <c r="C350" s="3"/>
-    </row>
-    <row r="351" spans="3:3">
+      <c r="D350" s="3"/>
+    </row>
+    <row r="351" spans="3:4">
       <c r="C351" s="3"/>
-    </row>
-    <row r="352" spans="3:3">
+      <c r="D351" s="3"/>
+    </row>
+    <row r="352" spans="3:4">
       <c r="C352" s="3"/>
-    </row>
-    <row r="353" spans="3:3">
+      <c r="D352" s="3"/>
+    </row>
+    <row r="353" spans="3:4">
       <c r="C353" s="3"/>
-    </row>
-    <row r="354" spans="3:3">
+      <c r="D353" s="3"/>
+    </row>
+    <row r="354" spans="3:4">
       <c r="C354" s="3"/>
-    </row>
-    <row r="355" spans="3:3">
+      <c r="D354" s="3"/>
+    </row>
+    <row r="355" spans="3:4">
       <c r="C355" s="3"/>
-    </row>
-    <row r="356" spans="3:3">
+      <c r="D355" s="3"/>
+    </row>
+    <row r="356" spans="3:4">
       <c r="C356" s="3"/>
-    </row>
-    <row r="357" spans="3:3">
+      <c r="D356" s="3"/>
+    </row>
+    <row r="357" spans="3:4">
       <c r="C357" s="3"/>
-    </row>
-    <row r="358" spans="3:3">
+      <c r="D357" s="3"/>
+    </row>
+    <row r="358" spans="3:4">
       <c r="C358" s="3"/>
-    </row>
-    <row r="359" spans="3:3">
+      <c r="D358" s="3"/>
+    </row>
+    <row r="359" spans="3:4">
       <c r="C359" s="3"/>
-    </row>
-    <row r="360" spans="3:3">
+      <c r="D359" s="3"/>
+    </row>
+    <row r="360" spans="3:4">
       <c r="C360" s="3"/>
-    </row>
-    <row r="361" spans="3:3">
+      <c r="D360" s="3"/>
+    </row>
+    <row r="361" spans="3:4">
       <c r="C361" s="3"/>
-    </row>
-    <row r="362" spans="3:3">
+      <c r="D361" s="3"/>
+    </row>
+    <row r="362" spans="3:4">
       <c r="C362" s="3"/>
-    </row>
-    <row r="363" spans="3:3">
+      <c r="D362" s="3"/>
+    </row>
+    <row r="363" spans="3:4">
       <c r="C363" s="3"/>
-    </row>
-    <row r="364" spans="3:3">
+      <c r="D363" s="3"/>
+    </row>
+    <row r="364" spans="3:4">
       <c r="C364" s="3"/>
-    </row>
-    <row r="365" spans="3:3">
+      <c r="D364" s="3"/>
+    </row>
+    <row r="365" spans="3:4">
       <c r="C365" s="3"/>
-    </row>
-    <row r="366" spans="3:3">
+      <c r="D365" s="3"/>
+    </row>
+    <row r="366" spans="3:4">
       <c r="C366" s="3"/>
-    </row>
-    <row r="367" spans="3:3">
+      <c r="D366" s="3"/>
+    </row>
+    <row r="367" spans="3:4">
       <c r="C367" s="3"/>
-    </row>
-    <row r="368" spans="3:3">
+      <c r="D367" s="3"/>
+    </row>
+    <row r="368" spans="3:4">
       <c r="C368" s="3"/>
-    </row>
-    <row r="369" spans="3:3">
+      <c r="D368" s="3"/>
+    </row>
+    <row r="369" spans="3:4">
       <c r="C369" s="3"/>
-    </row>
-    <row r="370" spans="3:3">
+      <c r="D369" s="3"/>
+    </row>
+    <row r="370" spans="3:4">
       <c r="C370" s="3"/>
-    </row>
-    <row r="371" spans="3:3">
+      <c r="D370" s="3"/>
+    </row>
+    <row r="371" spans="3:4">
       <c r="C371" s="3"/>
-    </row>
-    <row r="372" spans="3:3">
+      <c r="D371" s="3"/>
+    </row>
+    <row r="372" spans="3:4">
       <c r="C372" s="3"/>
-    </row>
-    <row r="373" spans="3:3">
+      <c r="D372" s="3"/>
+    </row>
+    <row r="373" spans="3:4">
       <c r="C373" s="3"/>
-    </row>
-    <row r="374" spans="3:3">
+      <c r="D373" s="3"/>
+    </row>
+    <row r="374" spans="3:4">
       <c r="C374" s="3"/>
-    </row>
-    <row r="375" spans="3:3">
+      <c r="D374" s="3"/>
+    </row>
+    <row r="375" spans="3:4">
       <c r="C375" s="3"/>
-    </row>
-    <row r="376" spans="3:3">
+      <c r="D375" s="3"/>
+    </row>
+    <row r="376" spans="3:4">
       <c r="C376" s="3"/>
-    </row>
-    <row r="377" spans="3:3">
+      <c r="D376" s="3"/>
+    </row>
+    <row r="377" spans="3:4">
       <c r="C377" s="3"/>
-    </row>
-    <row r="378" spans="3:3">
+      <c r="D377" s="3"/>
+    </row>
+    <row r="378" spans="3:4">
       <c r="C378" s="3"/>
-    </row>
-    <row r="379" spans="3:3">
+      <c r="D378" s="3"/>
+    </row>
+    <row r="379" spans="3:4">
       <c r="C379" s="3"/>
-    </row>
-    <row r="380" spans="3:3">
+      <c r="D379" s="3"/>
+    </row>
+    <row r="380" spans="3:4">
       <c r="C380" s="3"/>
-    </row>
-    <row r="381" spans="3:3">
+      <c r="D380" s="3"/>
+    </row>
+    <row r="381" spans="3:4">
       <c r="C381" s="3"/>
-    </row>
-    <row r="382" spans="3:3">
+      <c r="D381" s="3"/>
+    </row>
+    <row r="382" spans="3:4">
       <c r="C382" s="3"/>
-    </row>
-    <row r="383" spans="3:3">
+      <c r="D382" s="3"/>
+    </row>
+    <row r="383" spans="3:4">
       <c r="C383" s="3"/>
-    </row>
-    <row r="384" spans="3:3">
+      <c r="D383" s="3"/>
+    </row>
+    <row r="384" spans="3:4">
       <c r="C384" s="3"/>
-    </row>
-    <row r="385" spans="3:3">
+      <c r="D384" s="3"/>
+    </row>
+    <row r="385" spans="3:4">
       <c r="C385" s="3"/>
-    </row>
-    <row r="386" spans="3:3">
+      <c r="D385" s="3"/>
+    </row>
+    <row r="386" spans="3:4">
       <c r="C386" s="3"/>
-    </row>
-    <row r="387" spans="3:3">
+      <c r="D386" s="3"/>
+    </row>
+    <row r="387" spans="3:4">
       <c r="C387" s="3"/>
-    </row>
-    <row r="388" spans="3:3">
+      <c r="D387" s="3"/>
+    </row>
+    <row r="388" spans="3:4">
       <c r="C388" s="3"/>
-    </row>
-    <row r="389" spans="3:3">
+      <c r="D388" s="3"/>
+    </row>
+    <row r="389" spans="3:4">
       <c r="C389" s="3"/>
-    </row>
-    <row r="390" spans="3:3">
+      <c r="D389" s="3"/>
+    </row>
+    <row r="390" spans="3:4">
       <c r="C390" s="3"/>
-    </row>
-    <row r="391" spans="3:3">
+      <c r="D390" s="3"/>
+    </row>
+    <row r="391" spans="3:4">
       <c r="C391" s="3"/>
-    </row>
-    <row r="392" spans="3:3">
+      <c r="D391" s="3"/>
+    </row>
+    <row r="392" spans="3:4">
       <c r="C392" s="3"/>
-    </row>
-    <row r="393" spans="3:3">
+      <c r="D392" s="3"/>
+    </row>
+    <row r="393" spans="3:4">
       <c r="C393" s="3"/>
-    </row>
-    <row r="394" spans="3:3">
+      <c r="D393" s="3"/>
+    </row>
+    <row r="394" spans="3:4">
       <c r="C394" s="3"/>
-    </row>
-    <row r="395" spans="3:3">
+      <c r="D394" s="3"/>
+    </row>
+    <row r="395" spans="3:4">
       <c r="C395" s="3"/>
-    </row>
-    <row r="396" spans="3:3">
+      <c r="D395" s="3"/>
+    </row>
+    <row r="396" spans="3:4">
       <c r="C396" s="3"/>
-    </row>
-    <row r="397" spans="3:3">
+      <c r="D396" s="3"/>
+    </row>
+    <row r="397" spans="3:4">
       <c r="C397" s="3"/>
-    </row>
-    <row r="398" spans="3:3">
+      <c r="D397" s="3"/>
+    </row>
+    <row r="398" spans="3:4">
       <c r="C398" s="3"/>
-    </row>
-    <row r="399" spans="3:3">
+      <c r="D398" s="3"/>
+    </row>
+    <row r="399" spans="3:4">
       <c r="C399" s="3"/>
-    </row>
-    <row r="400" spans="3:3">
+      <c r="D399" s="3"/>
+    </row>
+    <row r="400" spans="3:4">
       <c r="C400" s="3"/>
-    </row>
-    <row r="401" spans="3:3">
+      <c r="D400" s="3"/>
+    </row>
+    <row r="401" spans="3:4">
       <c r="C401" s="3"/>
-    </row>
-    <row r="402" spans="3:3">
+      <c r="D401" s="3"/>
+    </row>
+    <row r="402" spans="3:4">
       <c r="C402" s="3"/>
-    </row>
-    <row r="403" spans="3:3">
+      <c r="D402" s="3"/>
+    </row>
+    <row r="403" spans="3:4">
       <c r="C403" s="3"/>
-    </row>
-    <row r="404" spans="3:3">
+      <c r="D403" s="3"/>
+    </row>
+    <row r="404" spans="3:4">
       <c r="C404" s="3"/>
-    </row>
-    <row r="405" spans="3:3">
+      <c r="D404" s="3"/>
+    </row>
+    <row r="405" spans="3:4">
       <c r="C405" s="3"/>
-    </row>
-    <row r="406" spans="3:3">
+      <c r="D405" s="3"/>
+    </row>
+    <row r="406" spans="3:4">
       <c r="C406" s="3"/>
+      <c r="D406" s="3"/>
+    </row>
+    <row r="407" spans="3:4">
+      <c r="C407" s="3"/>
+      <c r="D407" s="3"/>
+    </row>
+    <row r="408" spans="3:4">
+      <c r="C408" s="3"/>
+      <c r="D408" s="3"/>
+    </row>
+    <row r="409" spans="3:4">
+      <c r="C409" s="3"/>
+      <c r="D409" s="3"/>
+    </row>
+    <row r="410" spans="3:4">
+      <c r="C410" s="3"/>
+      <c r="D410" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E37" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C43:C66">
-    <sortCondition ref="C43:C66"/>
+  <autoFilter ref="A1:F41" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C47:C70">
+    <sortCondition ref="C47:C70"/>
   </sortState>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.74791666666666667" right="0.74791666666666667" top="0.98402777777777772" bottom="0.98402777777777772" header="0.51180555555555551" footer="0.51180555555555551"/>

</xml_diff>

<commit_message>
Minor corrections in source of trait data
</commit_message>
<xml_diff>
--- a/source_data/Braconidae_traits.xlsx
+++ b/source_data/Braconidae_traits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D33E7AA-AF5C-8B40-8AAD-E63C5411E56B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F70E1383-3FE6-3D41-B3EC-7DBA94A9160E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28180" windowHeight="17460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Swedish data" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Swedish data'!$A$1:$F$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Swedish data'!$A$1:$F$42</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="99">
   <si>
     <t>Phytophage-parasitoid</t>
     <phoneticPr fontId="3"/>
@@ -350,6 +350,12 @@
   </si>
   <si>
     <t>Marsh (1988) [reared from branches infested with cerambycids)</t>
+  </si>
+  <si>
+    <t>Proteropinae</t>
+  </si>
+  <si>
+    <t>Parasitoids of sawfly larvae (Jasso-Martinez et al. 2022)</t>
   </si>
 </sst>
 </file>
@@ -822,7 +828,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -866,7 +872,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -888,7 +894,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I410"/>
+  <dimension ref="A1:I411"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="47.1640625" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="2" width="15.83203125" style="1" customWidth="1"/>
@@ -1867,45 +1873,47 @@
       </c>
       <c r="I37" s="15"/>
     </row>
-    <row r="38" spans="1:9" ht="14">
-      <c r="A38" s="7" t="s">
+    <row r="38" spans="1:9" ht="13" customHeight="1">
+      <c r="A38" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C38" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="I38" s="15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="14">
+      <c r="A39" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C39" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D39" s="6" t="s">
         <v>42</v>
-      </c>
-      <c r="E38" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="F38" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G38" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="H38" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="I38" s="15"/>
-    </row>
-    <row r="39" spans="1:9" ht="13" customHeight="1">
-      <c r="A39" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>43</v>
       </c>
       <c r="E39" s="7" t="s">
         <v>0</v>
@@ -1922,28 +1930,28 @@
       <c r="I39" s="15"/>
     </row>
     <row r="40" spans="1:9" ht="13" customHeight="1">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="E40" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E40" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="F40" s="6" t="s">
+      <c r="F40" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G40" s="6" t="s">
+      <c r="G40" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="H40" s="6" t="s">
+      <c r="H40" s="7" t="s">
         <v>6</v>
       </c>
       <c r="I40" s="15"/>
@@ -1956,10 +1964,10 @@
         <v>21</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E41" s="6" t="s">
         <v>0</v>
@@ -1983,16 +1991,16 @@
         <v>21</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>0</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>0</v>
@@ -2002,43 +2010,45 @@
       </c>
       <c r="I42" s="15"/>
     </row>
-    <row r="43" spans="1:9" ht="15">
+    <row r="43" spans="1:9" ht="13" customHeight="1">
       <c r="A43" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C43" s="7" t="s">
+      <c r="C43" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I43" s="15"/>
+    </row>
+    <row r="44" spans="1:9" ht="15">
+      <c r="A44" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C44" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="D43" s="7" t="s">
+      <c r="D44" s="7" t="s">
         <v>52</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="G43" s="7"/>
-      <c r="H43" s="7"/>
-      <c r="I43" s="15" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="30">
-      <c r="A44" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B44" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C44" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>70</v>
       </c>
       <c r="E44" s="7" t="s">
         <v>53</v>
@@ -2046,14 +2056,10 @@
       <c r="F44" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="G44" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>6</v>
-      </c>
+      <c r="G44" s="7"/>
+      <c r="H44" s="7"/>
       <c r="I44" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="30">
@@ -2064,10 +2070,10 @@
         <v>21</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E45" s="7" t="s">
         <v>53</v>
@@ -2082,7 +2088,7 @@
         <v>6</v>
       </c>
       <c r="I45" s="15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="30">
@@ -2093,10 +2099,10 @@
         <v>21</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E46" s="7" t="s">
         <v>53</v>
@@ -2104,32 +2110,50 @@
       <c r="F46" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="G46" s="7" t="s">
+      <c r="G46" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I46" s="15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="30">
+      <c r="A47" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G47" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="H46" s="7" t="s">
+      <c r="H47" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="I46" s="15" t="s">
+      <c r="I47" s="15" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" ht="14">
-      <c r="A47" s="7"/>
-      <c r="B47" s="7"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="7"/>
-      <c r="F47" s="7"/>
-      <c r="G47" s="7"/>
-      <c r="H47" s="7"/>
-      <c r="I47" s="15"/>
     </row>
     <row r="48" spans="1:9" ht="14">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
-      <c r="C48" s="7"/>
-      <c r="D48" s="7"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
       <c r="E48" s="7"/>
       <c r="F48" s="7"/>
       <c r="G48" s="7"/>
@@ -2158,14 +2182,16 @@
       <c r="H50" s="7"/>
       <c r="I50" s="15"/>
     </row>
-    <row r="51" spans="1:9">
-      <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-      <c r="G51" s="5"/>
+    <row r="51" spans="1:9" ht="14">
+      <c r="A51" s="7"/>
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="15"/>
     </row>
     <row r="52" spans="1:9">
       <c r="A52" s="3"/>
@@ -2215,6 +2241,11 @@
     <row r="57" spans="1:9">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+      <c r="G57" s="5"/>
     </row>
     <row r="58" spans="1:9">
       <c r="A58" s="3"/>
@@ -2268,15 +2299,15 @@
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
     </row>
-    <row r="71" spans="1:4" ht="14">
+    <row r="71" spans="1:4">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
-      <c r="C71" s="2"/>
-      <c r="D71" s="2"/>
-    </row>
-    <row r="72" spans="1:4">
+    </row>
+    <row r="72" spans="1:4" ht="14">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
+      <c r="C72" s="2"/>
+      <c r="D72" s="2"/>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="3"/>
@@ -2310,17 +2341,17 @@
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
     </row>
-    <row r="81" spans="1:8" ht="14">
+    <row r="81" spans="1:8">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
-      <c r="E81" s="2"/>
-      <c r="F81" s="2"/>
-      <c r="G81" s="2"/>
-      <c r="H81" s="2"/>
-    </row>
-    <row r="82" spans="1:8">
+    </row>
+    <row r="82" spans="1:8" ht="14">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
+      <c r="E82" s="2"/>
+      <c r="F82" s="2"/>
+      <c r="G82" s="2"/>
+      <c r="H82" s="2"/>
     </row>
     <row r="83" spans="1:8">
       <c r="A83" s="3"/>
@@ -2354,27 +2385,27 @@
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
     </row>
-    <row r="91" spans="1:8" ht="14">
+    <row r="91" spans="1:8">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
-      <c r="E91" s="2"/>
-      <c r="F91" s="2"/>
-      <c r="G91" s="2"/>
-      <c r="H91" s="2"/>
-    </row>
-    <row r="92" spans="1:8">
+    </row>
+    <row r="92" spans="1:8" ht="14">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
-    </row>
-    <row r="93" spans="1:8" ht="14">
+      <c r="E92" s="2"/>
+      <c r="F92" s="2"/>
+      <c r="G92" s="2"/>
+      <c r="H92" s="2"/>
+    </row>
+    <row r="93" spans="1:8">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
-      <c r="C93" s="2"/>
-      <c r="D93" s="2"/>
-    </row>
-    <row r="94" spans="1:8">
+    </row>
+    <row r="94" spans="1:8" ht="14">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
+      <c r="C94" s="2"/>
+      <c r="D94" s="2"/>
     </row>
     <row r="95" spans="1:8">
       <c r="A95" s="3"/>
@@ -2396,17 +2427,15 @@
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
     </row>
-    <row r="100" spans="1:4" ht="14">
+    <row r="100" spans="1:4">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
-      <c r="C100" s="4"/>
-      <c r="D100" s="4"/>
     </row>
     <row r="101" spans="1:4" ht="14">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
-      <c r="C101" s="2"/>
-      <c r="D101" s="2"/>
+      <c r="C101" s="4"/>
+      <c r="D101" s="4"/>
     </row>
     <row r="102" spans="1:4" ht="14">
       <c r="A102" s="3"/>
@@ -2414,9 +2443,11 @@
       <c r="C102" s="2"/>
       <c r="D102" s="2"/>
     </row>
-    <row r="103" spans="1:4">
+    <row r="103" spans="1:4" ht="14">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
+      <c r="C103" s="2"/>
+      <c r="D103" s="2"/>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="3"/>
@@ -2530,15 +2561,15 @@
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
     </row>
-    <row r="132" spans="1:8" ht="14">
+    <row r="132" spans="1:8">
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
-      <c r="C132" s="2"/>
-      <c r="D132" s="2"/>
-    </row>
-    <row r="133" spans="1:8">
+    </row>
+    <row r="133" spans="1:8" ht="14">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
+      <c r="C133" s="2"/>
+      <c r="D133" s="2"/>
     </row>
     <row r="134" spans="1:8">
       <c r="A134" s="3"/>
@@ -2564,31 +2595,31 @@
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
     </row>
-    <row r="140" spans="1:8" ht="14">
+    <row r="140" spans="1:8">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
-      <c r="E140" s="4"/>
-      <c r="F140" s="4"/>
-      <c r="G140" s="4"/>
-      <c r="H140" s="4"/>
     </row>
     <row r="141" spans="1:8" ht="14">
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
-      <c r="E141" s="2"/>
-      <c r="F141" s="2"/>
-      <c r="G141" s="2"/>
-      <c r="H141" s="2"/>
+      <c r="E141" s="4"/>
+      <c r="F141" s="4"/>
+      <c r="G141" s="4"/>
+      <c r="H141" s="4"/>
     </row>
     <row r="142" spans="1:8" ht="14">
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
-      <c r="C142" s="2"/>
-      <c r="D142" s="2"/>
-    </row>
-    <row r="143" spans="1:8">
+      <c r="E142" s="2"/>
+      <c r="F142" s="2"/>
+      <c r="G142" s="2"/>
+      <c r="H142" s="2"/>
+    </row>
+    <row r="143" spans="1:8" ht="14">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
+      <c r="C143" s="2"/>
+      <c r="D143" s="2"/>
     </row>
     <row r="144" spans="1:8">
       <c r="A144" s="3"/>
@@ -2622,33 +2653,33 @@
       <c r="A151" s="3"/>
       <c r="B151" s="3"/>
     </row>
-    <row r="152" spans="1:8" ht="14">
+    <row r="152" spans="1:8">
       <c r="A152" s="3"/>
       <c r="B152" s="3"/>
-      <c r="E152" s="2"/>
-      <c r="F152" s="2"/>
-      <c r="G152" s="2"/>
-      <c r="H152" s="2"/>
-    </row>
-    <row r="153" spans="1:8">
+    </row>
+    <row r="153" spans="1:8" ht="14">
       <c r="A153" s="3"/>
       <c r="B153" s="3"/>
+      <c r="E153" s="2"/>
+      <c r="F153" s="2"/>
+      <c r="G153" s="2"/>
+      <c r="H153" s="2"/>
     </row>
     <row r="154" spans="1:8">
       <c r="A154" s="3"/>
       <c r="B154" s="3"/>
     </row>
-    <row r="155" spans="1:8" ht="14">
+    <row r="155" spans="1:8">
       <c r="A155" s="3"/>
       <c r="B155" s="3"/>
-      <c r="E155" s="2"/>
-      <c r="F155" s="2"/>
-      <c r="G155" s="2"/>
-      <c r="H155" s="2"/>
-    </row>
-    <row r="156" spans="1:8">
+    </row>
+    <row r="156" spans="1:8" ht="14">
       <c r="A156" s="3"/>
       <c r="B156" s="3"/>
+      <c r="E156" s="2"/>
+      <c r="F156" s="2"/>
+      <c r="G156" s="2"/>
+      <c r="H156" s="2"/>
     </row>
     <row r="157" spans="1:8">
       <c r="A157" s="3"/>
@@ -2786,21 +2817,21 @@
       <c r="A190" s="3"/>
       <c r="B190" s="3"/>
     </row>
-    <row r="191" spans="1:4" ht="14">
+    <row r="191" spans="1:4">
       <c r="A191" s="3"/>
       <c r="B191" s="3"/>
-      <c r="C191" s="4"/>
-      <c r="D191" s="4"/>
     </row>
     <row r="192" spans="1:4" ht="14">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
-      <c r="C192" s="2"/>
-      <c r="D192" s="2"/>
-    </row>
-    <row r="193" spans="1:4">
+      <c r="C192" s="4"/>
+      <c r="D192" s="4"/>
+    </row>
+    <row r="193" spans="1:4" ht="14">
       <c r="A193" s="3"/>
       <c r="B193" s="3"/>
+      <c r="C193" s="2"/>
+      <c r="D193" s="2"/>
     </row>
     <row r="194" spans="1:4">
       <c r="A194" s="3"/>
@@ -2838,29 +2869,29 @@
       <c r="A202" s="3"/>
       <c r="B202" s="3"/>
     </row>
-    <row r="203" spans="1:4" ht="14">
+    <row r="203" spans="1:4">
       <c r="A203" s="3"/>
       <c r="B203" s="3"/>
-      <c r="C203" s="2"/>
-      <c r="D203" s="2"/>
-    </row>
-    <row r="204" spans="1:4">
+    </row>
+    <row r="204" spans="1:4" ht="14">
       <c r="A204" s="3"/>
       <c r="B204" s="3"/>
+      <c r="C204" s="2"/>
+      <c r="D204" s="2"/>
     </row>
     <row r="205" spans="1:4">
       <c r="A205" s="3"/>
       <c r="B205" s="3"/>
     </row>
-    <row r="206" spans="1:4" ht="14">
+    <row r="206" spans="1:4">
       <c r="A206" s="3"/>
       <c r="B206" s="3"/>
-      <c r="C206" s="2"/>
-      <c r="D206" s="2"/>
-    </row>
-    <row r="207" spans="1:4">
+    </row>
+    <row r="207" spans="1:4" ht="14">
       <c r="A207" s="3"/>
       <c r="B207" s="3"/>
+      <c r="C207" s="2"/>
+      <c r="D207" s="2"/>
     </row>
     <row r="208" spans="1:4">
       <c r="A208" s="3"/>
@@ -2897,8 +2928,6 @@
     <row r="216" spans="1:4">
       <c r="A216" s="3"/>
       <c r="B216" s="3"/>
-      <c r="C216" s="3"/>
-      <c r="D216" s="3"/>
     </row>
     <row r="217" spans="1:4">
       <c r="A217" s="3"/>
@@ -2931,6 +2960,8 @@
       <c r="D221" s="3"/>
     </row>
     <row r="222" spans="1:4">
+      <c r="A222" s="3"/>
+      <c r="B222" s="3"/>
       <c r="C222" s="3"/>
       <c r="D222" s="3"/>
     </row>
@@ -3686,10 +3717,14 @@
       <c r="C410" s="3"/>
       <c r="D410" s="3"/>
     </row>
+    <row r="411" spans="3:4">
+      <c r="C411" s="3"/>
+      <c r="D411" s="3"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F41" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C47:C70">
-    <sortCondition ref="C47:C70"/>
+  <autoFilter ref="A1:F42" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C48:C71">
+    <sortCondition ref="C48:C71"/>
   </sortState>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.74791666666666667" right="0.74791666666666667" top="0.98402777777777772" bottom="0.98402777777777772" header="0.51180555555555551" footer="0.51180555555555551"/>

</xml_diff>

<commit_message>
Changes in braconid data files with respect to Doryctinae taxa
</commit_message>
<xml_diff>
--- a/source_data/Braconidae_traits.xlsx
+++ b/source_data/Braconidae_traits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F70E1383-3FE6-3D41-B3EC-7DBA94A9160E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E423B3B-1091-214C-AA11-75CEB678C75D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28180" windowHeight="17460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Swedish data" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Swedish data'!$A$1:$F$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Swedish data'!$A$1:$F$39</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="95">
   <si>
     <t>Phytophage-parasitoid</t>
     <phoneticPr fontId="3"/>
@@ -331,31 +331,19 @@
     <t>Mesostoinae</t>
   </si>
   <si>
-    <t>Doryctinae_Monarea</t>
-  </si>
-  <si>
-    <t>Doryctinae_Nervellius</t>
-  </si>
-  <si>
     <t>Doryctinae_Ontsira</t>
   </si>
   <si>
-    <t>Doryctinae_Syngaster</t>
-  </si>
-  <si>
     <t>Wang &amp; Aparicio (2020)</t>
   </si>
   <si>
-    <t>Iqbal et al. (2006)</t>
-  </si>
-  <si>
-    <t>Marsh (1988) [reared from branches infested with cerambycids)</t>
-  </si>
-  <si>
     <t>Proteropinae</t>
   </si>
   <si>
     <t>Parasitoids of sawfly larvae (Jasso-Martinez et al. 2022)</t>
+  </si>
+  <si>
+    <t>Marsh (1988) [Nervellius; reared from branches infested with cerambycids], Iqbal et al. (2006) [Syngaster]</t>
   </si>
 </sst>
 </file>
@@ -828,7 +816,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -872,7 +860,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -894,7 +882,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I411"/>
+  <dimension ref="A1:I408"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="47.1640625" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="2" width="15.83203125" style="1" customWidth="1"/>
@@ -1272,9 +1260,15 @@
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="15"/>
+      <c r="G14" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="I14" s="15" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="15" spans="1:9" ht="13" customHeight="1">
       <c r="A15" s="6" t="s">
@@ -1286,11 +1280,15 @@
       <c r="C15" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="D15" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
+      <c r="D15" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>8</v>
+      </c>
       <c r="G15" s="6" t="s">
         <v>0</v>
       </c>
@@ -1298,10 +1296,10 @@
         <v>8</v>
       </c>
       <c r="I15" s="15" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="13" customHeight="1">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="28" customHeight="1">
       <c r="A16" s="6" t="s">
         <v>17</v>
       </c>
@@ -1311,11 +1309,15 @@
       <c r="C16" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="D16" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
+      <c r="D16" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="G16" s="6" t="s">
         <v>0</v>
       </c>
@@ -1334,19 +1336,25 @@
         <v>21</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="D17" s="14" t="s">
-        <v>93</v>
+        <v>30</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>6</v>
       </c>
       <c r="G17" s="6" t="s">
         <v>0</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>95</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="13" customHeight="1">
@@ -1357,26 +1365,24 @@
         <v>21</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>88</v>
+        <v>31</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="E18" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G18" s="6" t="s">
+      <c r="F18" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G18" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="H18" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I18" s="15" t="s">
-        <v>69</v>
-      </c>
+      <c r="H18" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="I18" s="15"/>
     </row>
     <row r="19" spans="1:9" ht="13" customHeight="1">
       <c r="A19" s="6" t="s">
@@ -1386,22 +1392,26 @@
         <v>21</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>53</v>
+        <v>5</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
+        <v>8</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>8</v>
+      </c>
       <c r="I19" s="15"/>
     </row>
-    <row r="20" spans="1:9" ht="15">
+    <row r="20" spans="1:9" ht="13" customHeight="1">
       <c r="A20" s="6" t="s">
         <v>17</v>
       </c>
@@ -1409,10 +1419,10 @@
         <v>21</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>5</v>
@@ -1426,9 +1436,7 @@
       <c r="H20" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I20" s="15" t="s">
-        <v>60</v>
-      </c>
+      <c r="I20" s="15"/>
     </row>
     <row r="21" spans="1:9" ht="13" customHeight="1">
       <c r="A21" s="6" t="s">
@@ -1438,24 +1446,26 @@
         <v>21</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="F21" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H21" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G21" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="I21" s="15"/>
+      <c r="I21" s="15" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="22" spans="1:9" ht="13" customHeight="1">
       <c r="A22" s="6" t="s">
@@ -1465,22 +1475,22 @@
         <v>21</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G22" s="6" t="s">
         <v>0</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I22" s="15"/>
     </row>
@@ -1492,23 +1502,19 @@
         <v>21</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H23" s="6" t="s">
-        <v>6</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
       <c r="I23" s="15"/>
     </row>
     <row r="24" spans="1:9" ht="13" customHeight="1">
@@ -1519,16 +1525,16 @@
         <v>21</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>0</v>
@@ -1536,36 +1542,32 @@
       <c r="H24" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I24" s="15" t="s">
-        <v>64</v>
-      </c>
+      <c r="I24" s="15"/>
     </row>
     <row r="25" spans="1:9" ht="13" customHeight="1">
       <c r="A25" s="6" t="s">
-        <v>17</v>
+        <v>81</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>35</v>
+        <v>82</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>35</v>
+        <v>82</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>1</v>
+        <v>53</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G25" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H25" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I25" s="15"/>
+        <v>53</v>
+      </c>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="15" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="26" spans="1:9" ht="13" customHeight="1">
       <c r="A26" s="6" t="s">
@@ -1575,10 +1577,10 @@
         <v>21</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>53</v>
@@ -1598,37 +1600,35 @@
         <v>21</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>36</v>
+        <v>89</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H27" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I27" s="15"/>
+        <v>53</v>
+      </c>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="15" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="28" spans="1:9" ht="13" customHeight="1">
       <c r="A28" s="6" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>53</v>
@@ -1638,9 +1638,7 @@
       </c>
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
-      <c r="I28" s="15" t="s">
-        <v>83</v>
-      </c>
+      <c r="I28" s="15"/>
     </row>
     <row r="29" spans="1:9" ht="13" customHeight="1">
       <c r="A29" s="6" t="s">
@@ -1650,10 +1648,10 @@
         <v>21</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>53</v>
@@ -1673,45 +1671,53 @@
         <v>21</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>89</v>
+        <v>37</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>84</v>
+        <v>37</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="15" t="s">
-        <v>85</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I30" s="15"/>
     </row>
     <row r="31" spans="1:9" ht="13" customHeight="1">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C31" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6"/>
-      <c r="I31" s="15"/>
+      <c r="C31" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="I31" s="15" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="32" spans="1:9" ht="13" customHeight="1">
       <c r="A32" s="6" t="s">
@@ -1721,19 +1727,23 @@
         <v>21</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6"/>
+        <v>9</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>6</v>
+      </c>
       <c r="I32" s="15"/>
     </row>
     <row r="33" spans="1:9" ht="13" customHeight="1">
@@ -1744,16 +1754,16 @@
         <v>21</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="G33" s="6" t="s">
         <v>0</v>
@@ -1764,33 +1774,31 @@
       <c r="I33" s="15"/>
     </row>
     <row r="34" spans="1:9" ht="13" customHeight="1">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C34" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D34" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E34" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F34" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G34" s="7" t="s">
+      <c r="C34" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E34" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="H34" s="7" t="s">
+      <c r="F34" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I34" s="15" t="s">
-        <v>54</v>
-      </c>
+      <c r="I34" s="15"/>
     </row>
     <row r="35" spans="1:9" ht="13" customHeight="1">
       <c r="A35" s="6" t="s">
@@ -1800,75 +1808,77 @@
         <v>21</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>39</v>
+        <v>92</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>39</v>
+        <v>92</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>1</v>
+        <v>73</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>9</v>
+        <v>74</v>
       </c>
       <c r="G35" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="I35" s="15" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="14">
+      <c r="A36" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E36" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="H35" s="6" t="s">
+      <c r="F36" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="H36" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="I35" s="15"/>
-    </row>
-    <row r="36" spans="1:9" ht="13" customHeight="1">
-      <c r="A36" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D36" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G36" s="6" t="s">
+      <c r="I36" s="15"/>
+    </row>
+    <row r="37" spans="1:9" ht="13" customHeight="1">
+      <c r="A37" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E37" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="H36" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I36" s="15"/>
-    </row>
-    <row r="37" spans="1:9" ht="13" customHeight="1">
-      <c r="A37" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E37" s="6" t="s">
+      <c r="F37" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="F37" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H37" s="6" t="s">
+      <c r="H37" s="7" t="s">
         <v>6</v>
       </c>
       <c r="I37" s="15"/>
@@ -1881,126 +1891,122 @@
         <v>21</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>97</v>
+        <v>44</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>97</v>
+        <v>44</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="I38" s="15" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="14">
-      <c r="A39" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="I38" s="15"/>
+    </row>
+    <row r="39" spans="1:9" ht="13" customHeight="1">
+      <c r="A39" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E39" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E39" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="F39" s="7" t="s">
+      <c r="F39" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G39" s="7" t="s">
+      <c r="G39" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="H39" s="7" t="s">
+      <c r="H39" s="6" t="s">
         <v>6</v>
       </c>
       <c r="I39" s="15"/>
     </row>
     <row r="40" spans="1:9" ht="13" customHeight="1">
-      <c r="A40" s="7" t="s">
+      <c r="A40" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="E40" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E40" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="F40" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G40" s="7" t="s">
+      <c r="F40" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="G40" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="H40" s="7" t="s">
+      <c r="H40" s="6" t="s">
         <v>6</v>
       </c>
       <c r="I40" s="15"/>
     </row>
-    <row r="41" spans="1:9" ht="13" customHeight="1">
+    <row r="41" spans="1:9" ht="15">
       <c r="A41" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C41" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G41" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H41" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I41" s="15"/>
-    </row>
-    <row r="42" spans="1:9" ht="13" customHeight="1">
-      <c r="A42" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="D42" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>14</v>
+      <c r="C41" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G41" s="7"/>
+      <c r="H41" s="7"/>
+      <c r="I41" s="15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="30">
+      <c r="A42" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>53</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>0</v>
@@ -2008,26 +2014,28 @@
       <c r="H42" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I42" s="15"/>
-    </row>
-    <row r="43" spans="1:9" ht="13" customHeight="1">
-      <c r="A43" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>6</v>
+      <c r="I42" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="30">
+      <c r="A43" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>53</v>
       </c>
       <c r="G43" s="6" t="s">
         <v>0</v>
@@ -2035,20 +2043,22 @@
       <c r="H43" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I43" s="15"/>
-    </row>
-    <row r="44" spans="1:9" ht="15">
-      <c r="A44" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B44" s="6" t="s">
+      <c r="I43" s="15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="30">
+      <c r="A44" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B44" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="E44" s="7" t="s">
         <v>53</v>
@@ -2056,144 +2066,88 @@
       <c r="F44" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="G44" s="7"/>
-      <c r="H44" s="7"/>
+      <c r="G44" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="H44" s="7" t="s">
+        <v>74</v>
+      </c>
       <c r="I44" s="15" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" ht="30">
-      <c r="A45" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B45" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C45" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D45" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="E45" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F45" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="G45" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H45" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I45" s="15" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="30">
-      <c r="A46" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B46" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C46" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D46" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="E46" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F46" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="G46" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I46" s="15" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="30">
-      <c r="A47" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B47" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C47" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="D47" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E47" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F47" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="G47" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="H47" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="I47" s="15" t="s">
         <v>75</v>
       </c>
+    </row>
+    <row r="45" spans="1:9" ht="14">
+      <c r="A45" s="7"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="15"/>
+    </row>
+    <row r="46" spans="1:9" ht="14">
+      <c r="A46" s="7"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
+      <c r="H46" s="7"/>
+      <c r="I46" s="15"/>
+    </row>
+    <row r="47" spans="1:9" ht="14">
+      <c r="A47" s="7"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="7"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="15"/>
     </row>
     <row r="48" spans="1:9" ht="14">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
       <c r="E48" s="7"/>
       <c r="F48" s="7"/>
       <c r="G48" s="7"/>
       <c r="H48" s="7"/>
       <c r="I48" s="15"/>
     </row>
-    <row r="49" spans="1:9" ht="14">
-      <c r="A49" s="7"/>
-      <c r="B49" s="7"/>
-      <c r="C49" s="7"/>
-      <c r="D49" s="7"/>
-      <c r="E49" s="7"/>
-      <c r="F49" s="7"/>
-      <c r="G49" s="7"/>
-      <c r="H49" s="7"/>
-      <c r="I49" s="15"/>
-    </row>
-    <row r="50" spans="1:9" ht="14">
-      <c r="A50" s="7"/>
-      <c r="B50" s="7"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="7"/>
-      <c r="F50" s="7"/>
-      <c r="G50" s="7"/>
-      <c r="H50" s="7"/>
-      <c r="I50" s="15"/>
-    </row>
-    <row r="51" spans="1:9" ht="14">
-      <c r="A51" s="7"/>
-      <c r="B51" s="7"/>
-      <c r="C51" s="7"/>
-      <c r="D51" s="7"/>
-      <c r="E51" s="7"/>
-      <c r="F51" s="7"/>
-      <c r="G51" s="7"/>
-      <c r="H51" s="7"/>
-      <c r="I51" s="15"/>
-    </row>
-    <row r="52" spans="1:9">
+    <row r="49" spans="1:7">
+      <c r="A49" s="3"/>
+      <c r="B49" s="3"/>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50" s="3"/>
+      <c r="B50" s="3"/>
+      <c r="C50" s="5"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="5"/>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51" s="3"/>
+      <c r="B51" s="3"/>
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+    </row>
+    <row r="52" spans="1:7">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="5"/>
@@ -2202,7 +2156,7 @@
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
     </row>
-    <row r="53" spans="1:9">
+    <row r="53" spans="1:7">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="5"/>
@@ -2211,7 +2165,7 @@
       <c r="F53" s="5"/>
       <c r="G53" s="5"/>
     </row>
-    <row r="54" spans="1:9">
+    <row r="54" spans="1:7">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="5"/>
@@ -2220,124 +2174,113 @@
       <c r="F54" s="5"/>
       <c r="G54" s="5"/>
     </row>
-    <row r="55" spans="1:9">
+    <row r="55" spans="1:7">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5"/>
-    </row>
-    <row r="56" spans="1:9">
+    </row>
+    <row r="56" spans="1:7">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="5"/>
-      <c r="E56" s="5"/>
-      <c r="F56" s="5"/>
-      <c r="G56" s="5"/>
-    </row>
-    <row r="57" spans="1:9">
+    </row>
+    <row r="57" spans="1:7">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
-      <c r="C57" s="5"/>
-      <c r="D57" s="5"/>
-      <c r="E57" s="5"/>
-      <c r="F57" s="5"/>
-      <c r="G57" s="5"/>
-    </row>
-    <row r="58" spans="1:9">
+    </row>
+    <row r="58" spans="1:7">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
     </row>
-    <row r="59" spans="1:9">
+    <row r="59" spans="1:7">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
     </row>
-    <row r="60" spans="1:9">
+    <row r="60" spans="1:7">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
     </row>
-    <row r="61" spans="1:9">
+    <row r="61" spans="1:7">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
     </row>
-    <row r="62" spans="1:9">
+    <row r="62" spans="1:7">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
     </row>
-    <row r="63" spans="1:9">
+    <row r="63" spans="1:7">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
     </row>
-    <row r="64" spans="1:9">
+    <row r="64" spans="1:7">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
     </row>
-    <row r="65" spans="1:4">
+    <row r="65" spans="1:8">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
     </row>
-    <row r="66" spans="1:4">
+    <row r="66" spans="1:8">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
     </row>
-    <row r="67" spans="1:4">
+    <row r="67" spans="1:8">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
     </row>
-    <row r="68" spans="1:4">
+    <row r="68" spans="1:8">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
     </row>
-    <row r="69" spans="1:4">
+    <row r="69" spans="1:8" ht="14">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
-    </row>
-    <row r="70" spans="1:4">
+      <c r="C69" s="2"/>
+      <c r="D69" s="2"/>
+    </row>
+    <row r="70" spans="1:8">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
     </row>
-    <row r="71" spans="1:4">
+    <row r="71" spans="1:8">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
     </row>
-    <row r="72" spans="1:4" ht="14">
+    <row r="72" spans="1:8">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
-      <c r="C72" s="2"/>
-      <c r="D72" s="2"/>
-    </row>
-    <row r="73" spans="1:4">
+    </row>
+    <row r="73" spans="1:8">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
     </row>
-    <row r="74" spans="1:4">
+    <row r="74" spans="1:8">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
     </row>
-    <row r="75" spans="1:4">
+    <row r="75" spans="1:8">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
     </row>
-    <row r="76" spans="1:4">
+    <row r="76" spans="1:8">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
     </row>
-    <row r="77" spans="1:4">
+    <row r="77" spans="1:8">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
     </row>
-    <row r="78" spans="1:4">
+    <row r="78" spans="1:8">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
     </row>
-    <row r="79" spans="1:4">
+    <row r="79" spans="1:8" ht="14">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
-    </row>
-    <row r="80" spans="1:4">
+      <c r="E79" s="2"/>
+      <c r="F79" s="2"/>
+      <c r="G79" s="2"/>
+      <c r="H79" s="2"/>
+    </row>
+    <row r="80" spans="1:8">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
     </row>
@@ -2345,13 +2288,9 @@
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
     </row>
-    <row r="82" spans="1:8" ht="14">
+    <row r="82" spans="1:8">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
-      <c r="E82" s="2"/>
-      <c r="F82" s="2"/>
-      <c r="G82" s="2"/>
-      <c r="H82" s="2"/>
     </row>
     <row r="83" spans="1:8">
       <c r="A83" s="3"/>
@@ -2377,35 +2316,35 @@
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
     </row>
-    <row r="89" spans="1:8">
+    <row r="89" spans="1:8" ht="14">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
+      <c r="E89" s="2"/>
+      <c r="F89" s="2"/>
+      <c r="G89" s="2"/>
+      <c r="H89" s="2"/>
     </row>
     <row r="90" spans="1:8">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
     </row>
-    <row r="91" spans="1:8">
+    <row r="91" spans="1:8" ht="14">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
-    </row>
-    <row r="92" spans="1:8" ht="14">
+      <c r="C91" s="2"/>
+      <c r="D91" s="2"/>
+    </row>
+    <row r="92" spans="1:8">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
-      <c r="E92" s="2"/>
-      <c r="F92" s="2"/>
-      <c r="G92" s="2"/>
-      <c r="H92" s="2"/>
     </row>
     <row r="93" spans="1:8">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
     </row>
-    <row r="94" spans="1:8" ht="14">
+    <row r="94" spans="1:8">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
-      <c r="C94" s="2"/>
-      <c r="D94" s="2"/>
     </row>
     <row r="95" spans="1:8">
       <c r="A95" s="3"/>
@@ -2419,35 +2358,35 @@
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
     </row>
-    <row r="98" spans="1:4">
+    <row r="98" spans="1:4" ht="14">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
-    </row>
-    <row r="99" spans="1:4">
+      <c r="C98" s="4"/>
+      <c r="D98" s="4"/>
+    </row>
+    <row r="99" spans="1:4" ht="14">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
-    </row>
-    <row r="100" spans="1:4">
+      <c r="C99" s="2"/>
+      <c r="D99" s="2"/>
+    </row>
+    <row r="100" spans="1:4" ht="14">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
-    </row>
-    <row r="101" spans="1:4" ht="14">
+      <c r="C100" s="2"/>
+      <c r="D100" s="2"/>
+    </row>
+    <row r="101" spans="1:4">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
-      <c r="C101" s="4"/>
-      <c r="D101" s="4"/>
-    </row>
-    <row r="102" spans="1:4" ht="14">
+    </row>
+    <row r="102" spans="1:4">
       <c r="A102" s="3"/>
       <c r="B102" s="3"/>
-      <c r="C102" s="2"/>
-      <c r="D102" s="2"/>
-    </row>
-    <row r="103" spans="1:4" ht="14">
+    </row>
+    <row r="103" spans="1:4">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
-      <c r="C103" s="2"/>
-      <c r="D103" s="2"/>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="3"/>
@@ -2553,9 +2492,11 @@
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
     </row>
-    <row r="130" spans="1:8">
+    <row r="130" spans="1:8" ht="14">
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
+      <c r="C130" s="2"/>
+      <c r="D130" s="2"/>
     </row>
     <row r="131" spans="1:8">
       <c r="A131" s="3"/>
@@ -2565,11 +2506,9 @@
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
     </row>
-    <row r="133" spans="1:8" ht="14">
+    <row r="133" spans="1:8">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
-      <c r="C133" s="2"/>
-      <c r="D133" s="2"/>
     </row>
     <row r="134" spans="1:8">
       <c r="A134" s="3"/>
@@ -2587,39 +2526,39 @@
       <c r="A137" s="3"/>
       <c r="B137" s="3"/>
     </row>
-    <row r="138" spans="1:8">
+    <row r="138" spans="1:8" ht="14">
       <c r="A138" s="3"/>
       <c r="B138" s="3"/>
-    </row>
-    <row r="139" spans="1:8">
+      <c r="E138" s="4"/>
+      <c r="F138" s="4"/>
+      <c r="G138" s="4"/>
+      <c r="H138" s="4"/>
+    </row>
+    <row r="139" spans="1:8" ht="14">
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
-    </row>
-    <row r="140" spans="1:8">
+      <c r="E139" s="2"/>
+      <c r="F139" s="2"/>
+      <c r="G139" s="2"/>
+      <c r="H139" s="2"/>
+    </row>
+    <row r="140" spans="1:8" ht="14">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
-    </row>
-    <row r="141" spans="1:8" ht="14">
+      <c r="C140" s="2"/>
+      <c r="D140" s="2"/>
+    </row>
+    <row r="141" spans="1:8">
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
-      <c r="E141" s="4"/>
-      <c r="F141" s="4"/>
-      <c r="G141" s="4"/>
-      <c r="H141" s="4"/>
-    </row>
-    <row r="142" spans="1:8" ht="14">
+    </row>
+    <row r="142" spans="1:8">
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
-      <c r="E142" s="2"/>
-      <c r="F142" s="2"/>
-      <c r="G142" s="2"/>
-      <c r="H142" s="2"/>
-    </row>
-    <row r="143" spans="1:8" ht="14">
+    </row>
+    <row r="143" spans="1:8">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
-      <c r="C143" s="2"/>
-      <c r="D143" s="2"/>
     </row>
     <row r="144" spans="1:8">
       <c r="A144" s="3"/>
@@ -2645,9 +2584,13 @@
       <c r="A149" s="3"/>
       <c r="B149" s="3"/>
     </row>
-    <row r="150" spans="1:8">
+    <row r="150" spans="1:8" ht="14">
       <c r="A150" s="3"/>
       <c r="B150" s="3"/>
+      <c r="E150" s="2"/>
+      <c r="F150" s="2"/>
+      <c r="G150" s="2"/>
+      <c r="H150" s="2"/>
     </row>
     <row r="151" spans="1:8">
       <c r="A151" s="3"/>
@@ -2673,13 +2616,9 @@
       <c r="A155" s="3"/>
       <c r="B155" s="3"/>
     </row>
-    <row r="156" spans="1:8" ht="14">
+    <row r="156" spans="1:8">
       <c r="A156" s="3"/>
       <c r="B156" s="3"/>
-      <c r="E156" s="2"/>
-      <c r="F156" s="2"/>
-      <c r="G156" s="2"/>
-      <c r="H156" s="2"/>
     </row>
     <row r="157" spans="1:8">
       <c r="A157" s="3"/>
@@ -2809,29 +2748,29 @@
       <c r="A188" s="3"/>
       <c r="B188" s="3"/>
     </row>
-    <row r="189" spans="1:4">
+    <row r="189" spans="1:4" ht="14">
       <c r="A189" s="3"/>
       <c r="B189" s="3"/>
-    </row>
-    <row r="190" spans="1:4">
+      <c r="C189" s="4"/>
+      <c r="D189" s="4"/>
+    </row>
+    <row r="190" spans="1:4" ht="14">
       <c r="A190" s="3"/>
       <c r="B190" s="3"/>
+      <c r="C190" s="2"/>
+      <c r="D190" s="2"/>
     </row>
     <row r="191" spans="1:4">
       <c r="A191" s="3"/>
       <c r="B191" s="3"/>
     </row>
-    <row r="192" spans="1:4" ht="14">
+    <row r="192" spans="1:4">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
-      <c r="C192" s="4"/>
-      <c r="D192" s="4"/>
-    </row>
-    <row r="193" spans="1:4" ht="14">
+    </row>
+    <row r="193" spans="1:4">
       <c r="A193" s="3"/>
       <c r="B193" s="3"/>
-      <c r="C193" s="2"/>
-      <c r="D193" s="2"/>
     </row>
     <row r="194" spans="1:4">
       <c r="A194" s="3"/>
@@ -2861,9 +2800,11 @@
       <c r="A200" s="3"/>
       <c r="B200" s="3"/>
     </row>
-    <row r="201" spans="1:4">
+    <row r="201" spans="1:4" ht="14">
       <c r="A201" s="3"/>
       <c r="B201" s="3"/>
+      <c r="C201" s="2"/>
+      <c r="D201" s="2"/>
     </row>
     <row r="202" spans="1:4">
       <c r="A202" s="3"/>
@@ -2887,11 +2828,9 @@
       <c r="A206" s="3"/>
       <c r="B206" s="3"/>
     </row>
-    <row r="207" spans="1:4" ht="14">
+    <row r="207" spans="1:4">
       <c r="A207" s="3"/>
       <c r="B207" s="3"/>
-      <c r="C207" s="2"/>
-      <c r="D207" s="2"/>
     </row>
     <row r="208" spans="1:4">
       <c r="A208" s="3"/>
@@ -2920,14 +2859,20 @@
     <row r="214" spans="1:4">
       <c r="A214" s="3"/>
       <c r="B214" s="3"/>
+      <c r="C214" s="3"/>
+      <c r="D214" s="3"/>
     </row>
     <row r="215" spans="1:4">
       <c r="A215" s="3"/>
       <c r="B215" s="3"/>
+      <c r="C215" s="3"/>
+      <c r="D215" s="3"/>
     </row>
     <row r="216" spans="1:4">
       <c r="A216" s="3"/>
       <c r="B216" s="3"/>
+      <c r="C216" s="3"/>
+      <c r="D216" s="3"/>
     </row>
     <row r="217" spans="1:4">
       <c r="A217" s="3"/>
@@ -2948,20 +2893,14 @@
       <c r="D219" s="3"/>
     </row>
     <row r="220" spans="1:4">
-      <c r="A220" s="3"/>
-      <c r="B220" s="3"/>
       <c r="C220" s="3"/>
       <c r="D220" s="3"/>
     </row>
     <row r="221" spans="1:4">
-      <c r="A221" s="3"/>
-      <c r="B221" s="3"/>
       <c r="C221" s="3"/>
       <c r="D221" s="3"/>
     </row>
     <row r="222" spans="1:4">
-      <c r="A222" s="3"/>
-      <c r="B222" s="3"/>
       <c r="C222" s="3"/>
       <c r="D222" s="3"/>
     </row>
@@ -3709,22 +3648,10 @@
       <c r="C408" s="3"/>
       <c r="D408" s="3"/>
     </row>
-    <row r="409" spans="3:4">
-      <c r="C409" s="3"/>
-      <c r="D409" s="3"/>
-    </row>
-    <row r="410" spans="3:4">
-      <c r="C410" s="3"/>
-      <c r="D410" s="3"/>
-    </row>
-    <row r="411" spans="3:4">
-      <c r="C411" s="3"/>
-      <c r="D411" s="3"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F42" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C48:C71">
-    <sortCondition ref="C48:C71"/>
+  <autoFilter ref="A1:F39" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C45:C68">
+    <sortCondition ref="C45:C68"/>
   </sortState>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.74791666666666667" right="0.74791666666666667" top="0.98402777777777772" bottom="0.98402777777777772" header="0.51180555555555551" footer="0.51180555555555551"/>

</xml_diff>

<commit_message>
Updated Braconidae traits data. Added braconid references to the README file
</commit_message>
<xml_diff>
--- a/source_data/Braconidae_traits.xlsx
+++ b/source_data/Braconidae_traits.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E423B3B-1091-214C-AA11-75CEB678C75D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12162A83-17C5-244E-BB48-CF1DA02E9F6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28180" windowHeight="17460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="17380" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Swedish data" sheetId="1" r:id="rId1"/>
+    <sheet name="Trait data" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Swedish data'!$A$1:$F$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Trait data'!$A$1:$F$42</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="108">
   <si>
     <t>Phytophage-parasitoid</t>
     <phoneticPr fontId="3"/>
@@ -223,9 +223,6 @@
     <t>NA</t>
   </si>
   <si>
-    <t>Not officially reported from Sweden but prob present</t>
-  </si>
-  <si>
     <t>Includes Adeliini, formerly separate subfamily</t>
   </si>
   <si>
@@ -286,24 +283,9 @@
     <t>Plants</t>
   </si>
   <si>
-    <t>Apparently restricted to SE Asia, Oriental region, New Guinea. Two genera: Xiphozele and Distilirella</t>
-  </si>
-  <si>
     <t>Includes Cercobarconinae; life history unknown</t>
   </si>
   <si>
-    <t>Occurs in Madagascar but no verified GenBank CO1 sequences</t>
-  </si>
-  <si>
-    <t>One species reared from Ectoedemia phleophaga (Quicke 2015); no nucleotide sequences in GenBank</t>
-  </si>
-  <si>
-    <t>No nucleotide sequences in GenBank</t>
-  </si>
-  <si>
-    <t>Only an unverified mitochondrial genome in GenBank</t>
-  </si>
-  <si>
     <t>Hymrnoptera</t>
   </si>
   <si>
@@ -331,26 +313,262 @@
     <t>Mesostoinae</t>
   </si>
   <si>
+    <t>Doryctinae_Monarea</t>
+  </si>
+  <si>
+    <t>Doryctinae_Nervellius</t>
+  </si>
+  <si>
     <t>Doryctinae_Ontsira</t>
   </si>
   <si>
+    <t>Doryctinae_Syngaster</t>
+  </si>
+  <si>
     <t>Wang &amp; Aparicio (2020)</t>
   </si>
   <si>
+    <t>Iqbal et al. (2006)</t>
+  </si>
+  <si>
+    <t>Marsh (1988) [reared from branches infested with cerambycids)</t>
+  </si>
+  <si>
     <t>Proteropinae</t>
   </si>
   <si>
     <t>Parasitoids of sawfly larvae (Jasso-Martinez et al. 2022)</t>
   </si>
   <si>
-    <t>Marsh (1988) [Nervellius; reared from branches infested with cerambycids], Iqbal et al. (2006) [Syngaster]</t>
+    <r>
+      <t xml:space="preserve">The North American genus </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Urosigalphus </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">is a prasitoid of seed feeding beetles (Curculionidae &amp; Brucinae) (Arias Penna &amp; Whitfield 2012). Host records of african species unknown, but the african genus </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Afrocampsis </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>has been proposed by M. Sharkey to be a parasitoid of wood or seed feeding beetles based on morphological characters (Quicke et al. 2002).</t>
+    </r>
+  </si>
+  <si>
+    <t>The majority are parasitoids of saprophagous hosts (all in the tribe Alysiini). However, many are also parasitoids of leaf mining Diptera (all members of the tribe Dacnusini and a few Alysiini). All hosts are cyclorrhaphous Diptera (Shaw &amp; Huddleston, 1991).</t>
+  </si>
+  <si>
+    <t>Only an unverified mitochondrial genome in GenBank. Contains only one species from Chile. Hosts unkown but thought to be konobiont ectoparasitoids of xylophagous Coleoptera based on morphology and phylogenetic placement. (Sharkey 1997).</t>
+  </si>
+  <si>
+    <t>Wood</t>
+  </si>
+  <si>
+    <t>Most are egg-larval parasitoids of phytophagous Coleoptera (e.g., Curculionidae), some attack wood-boring Coleoptera larvae (e.g., Cerembycidae). Some Blacini have been proposed to be parasitoids of saprophagous Coleoptera based on the habitats they have been caught in, but they have never been reared. Hosts summarized by Shaw &amp; Huddleston (1991) and Ghahari et al. (2022)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">No nucleotide sequences in GenBank. Two species reared from larval </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Boreus</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Mecoptera), feeding on moss (Mason 1976).</t>
+    </r>
+  </si>
+  <si>
+    <t>Parasitoids of leaf mining insects, predominantly Lepidoptera and Tenthredinidae (van Achterberg 1983).</t>
+  </si>
+  <si>
+    <t>Hosts unknown, but has been speculated based on multiple morphological characters to be a parasitoid of wood-, stem-, or possibly root-boring Lepidoptera (Sharkey et al. 2009).</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">South American subfamily. One species, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Epsilogaster bicolor,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> has been reared from a twig-boring Lepidoptera, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Cephalanthus occidentalis</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Whitfield &amp; Mason 1994)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Meteoridea hutsoni </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">is a parasitoid of the leaf rolling lepidopteran  </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Opisina arenosella</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>, Biology studied by Ghosh &amp; Abdurahiman (1984).</t>
+    </r>
+  </si>
+  <si>
+    <t>Not officially reported from Sweden but several records are known.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">One species reared from </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Ectoedemia phleophaga</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Quicke 2015); no nucleotide sequences in GenBank</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Apparently restricted to SE Asia, Oriental region, New Guinea. Two genera: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Xiphozele</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Distilirella</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Occurs in Madagascar but no verified GenBank CO1 sequences. Parasitoids of plant boring Lepidoptera (Achterberg 1979)</t>
+  </si>
+  <si>
+    <t>South American genus (Belokoblylskij et al. 2014).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -434,6 +652,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -471,11 +695,9 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -486,6 +708,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Default" xfId="1" xr:uid="{97A9FA61-B53C-564A-BB10-C00C98D42059}"/>
@@ -882,16 +1106,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I408"/>
+  <dimension ref="A1:I411"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="47.1640625" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="2" width="15.83203125" style="1" customWidth="1"/>
     <col min="3" max="4" width="31.5" style="1" customWidth="1"/>
     <col min="5" max="5" width="22.33203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="21.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="21.5" style="1" customWidth="1"/>
-    <col min="8" max="8" width="23" style="1" customWidth="1"/>
-    <col min="9" max="9" width="50.83203125" style="16" customWidth="1"/>
+    <col min="7" max="7" width="23.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="57.5" style="14" customWidth="1"/>
     <col min="10" max="16384" width="47.1640625" style="1"/>
   </cols>
   <sheetData>
@@ -906,45 +1130,52 @@
         <v>46</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="E1" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="15" t="s">
         <v>50</v>
       </c>
       <c r="I1" s="8" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="8" customFormat="1" ht="15">
-      <c r="A2" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="E2" s="12" t="s">
+    <row r="2" spans="1:9" s="8" customFormat="1" ht="90">
+      <c r="A2" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E2" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
+      <c r="G2" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="H2" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="I2" s="13" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="3" spans="1:9" ht="13" customHeight="1">
       <c r="A3" s="6" t="s">
@@ -971,9 +1202,9 @@
       <c r="H3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="15"/>
-    </row>
-    <row r="4" spans="1:9" ht="13" customHeight="1">
+      <c r="I3" s="13"/>
+    </row>
+    <row r="4" spans="1:9" ht="60" customHeight="1">
       <c r="A4" s="6" t="s">
         <v>17</v>
       </c>
@@ -998,7 +1229,9 @@
       <c r="H4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I4" s="15"/>
+      <c r="I4" s="13" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="5" spans="1:9" ht="14">
       <c r="A5" s="6" t="s">
@@ -1025,9 +1258,9 @@
       <c r="H5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I5" s="15"/>
-    </row>
-    <row r="6" spans="1:9" ht="15">
+      <c r="I5" s="13"/>
+    </row>
+    <row r="6" spans="1:9" ht="60">
       <c r="A6" s="6" t="s">
         <v>17</v>
       </c>
@@ -1035,10 +1268,10 @@
         <v>21</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>53</v>
@@ -1046,13 +1279,17 @@
       <c r="F6" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="15" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="14">
+      <c r="G6" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="88" customHeight="1">
       <c r="A7" s="6" t="s">
         <v>17</v>
       </c>
@@ -1060,26 +1297,28 @@
         <v>21</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>3</v>
+        <v>72</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>6</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>3</v>
+        <v>72</v>
       </c>
       <c r="H7" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="15"/>
-    </row>
-    <row r="8" spans="1:9" ht="15">
+      <c r="I7" s="13" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30">
       <c r="A8" s="6" t="s">
         <v>17</v>
       </c>
@@ -1087,25 +1326,25 @@
         <v>21</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>3</v>
+        <v>72</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>6</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>3</v>
+        <v>72</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="I8" s="15" t="s">
-        <v>79</v>
+      <c r="I8" s="13" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="13" customHeight="1">
@@ -1133,7 +1372,7 @@
       <c r="H9" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I9" s="15"/>
+      <c r="I9" s="13"/>
     </row>
     <row r="10" spans="1:9" ht="13" customHeight="1">
       <c r="A10" s="6" t="s">
@@ -1160,7 +1399,7 @@
       <c r="H10" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I10" s="15"/>
+      <c r="I10" s="13"/>
     </row>
     <row r="11" spans="1:9" ht="13" customHeight="1">
       <c r="A11" s="6" t="s">
@@ -1187,7 +1426,7 @@
       <c r="H11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I11" s="15"/>
+      <c r="I11" s="13"/>
     </row>
     <row r="12" spans="1:9" ht="13" customHeight="1">
       <c r="A12" s="6" t="s">
@@ -1214,7 +1453,7 @@
       <c r="H12" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="I12" s="15"/>
+      <c r="I12" s="13"/>
     </row>
     <row r="13" spans="1:9" ht="13" customHeight="1">
       <c r="A13" s="6" t="s">
@@ -1241,8 +1480,8 @@
       <c r="H13" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I13" s="15" t="s">
-        <v>55</v>
+      <c r="I13" s="13" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="13" customHeight="1">
@@ -1253,21 +1492,25 @@
         <v>21</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
+        <v>82</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="G14" s="6" t="s">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I14" s="15" t="s">
-        <v>91</v>
+        <v>53</v>
+      </c>
+      <c r="I14" s="13" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="13" customHeight="1">
@@ -1278,28 +1521,24 @@
         <v>21</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>8</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
       <c r="G15" s="6" t="s">
         <v>0</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I15" s="15" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="28" customHeight="1">
+      <c r="I15" s="13" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="13" customHeight="1">
       <c r="A16" s="6" t="s">
         <v>17</v>
       </c>
@@ -1307,25 +1546,21 @@
         <v>21</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>53</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
       <c r="G16" s="6" t="s">
         <v>0</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I16" s="15" t="s">
-        <v>94</v>
+      <c r="I16" s="13" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15">
@@ -1336,25 +1571,21 @@
         <v>21</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>6</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
       <c r="G17" s="6" t="s">
         <v>0</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I17" s="15" t="s">
-        <v>60</v>
+        <v>8</v>
+      </c>
+      <c r="I17" s="13" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="13" customHeight="1">
@@ -1365,24 +1596,26 @@
         <v>21</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>31</v>
+        <v>82</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="E18" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E18" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="G18" s="7" t="s">
+      <c r="F18" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G18" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="H18" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="I18" s="15"/>
+      <c r="H18" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="I18" s="13" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="19" spans="1:9" ht="13" customHeight="1">
       <c r="A19" s="6" t="s">
@@ -1392,26 +1625,22 @@
         <v>21</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>32</v>
+        <v>82</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H19" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I19" s="15"/>
-    </row>
-    <row r="20" spans="1:9" ht="13" customHeight="1">
+        <v>53</v>
+      </c>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="13"/>
+    </row>
+    <row r="20" spans="1:9" ht="15">
       <c r="A20" s="6" t="s">
         <v>17</v>
       </c>
@@ -1419,10 +1648,10 @@
         <v>21</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>5</v>
@@ -1436,9 +1665,11 @@
       <c r="H20" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I20" s="15"/>
-    </row>
-    <row r="21" spans="1:9" ht="13" customHeight="1">
+      <c r="I20" s="13" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="33" customHeight="1">
       <c r="A21" s="6" t="s">
         <v>17</v>
       </c>
@@ -1446,25 +1677,25 @@
         <v>21</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G21" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G21" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="H21" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="I21" s="15" t="s">
-        <v>64</v>
+      <c r="I21" s="13" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="13" customHeight="1">
@@ -1475,24 +1706,24 @@
         <v>21</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G22" s="6" t="s">
         <v>0</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I22" s="15"/>
+        <v>8</v>
+      </c>
+      <c r="I22" s="13"/>
     </row>
     <row r="23" spans="1:9" ht="13" customHeight="1">
       <c r="A23" s="6" t="s">
@@ -1502,20 +1733,24 @@
         <v>21</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>53</v>
+        <v>5</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="15"/>
+        <v>6</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I23" s="13"/>
     </row>
     <row r="24" spans="1:9" ht="13" customHeight="1">
       <c r="A24" s="6" t="s">
@@ -1525,16 +1760,16 @@
         <v>21</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>0</v>
@@ -1542,34 +1777,38 @@
       <c r="H24" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I24" s="15"/>
+      <c r="I24" s="13" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="25" spans="1:9" ht="13" customHeight="1">
       <c r="A25" s="6" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>82</v>
+        <v>35</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>82</v>
+        <v>35</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="15" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="13" customHeight="1">
+        <v>9</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I25" s="13"/>
+    </row>
+    <row r="26" spans="1:9" ht="47" customHeight="1">
       <c r="A26" s="6" t="s">
         <v>17</v>
       </c>
@@ -1577,10 +1816,10 @@
         <v>21</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>53</v>
@@ -1588,9 +1827,15 @@
       <c r="F26" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="15"/>
+      <c r="G26" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="I26" s="13" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="27" spans="1:9" ht="13" customHeight="1">
       <c r="A27" s="6" t="s">
@@ -1600,35 +1845,37 @@
         <v>21</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>89</v>
+        <v>36</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="15" t="s">
-        <v>85</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I27" s="13"/>
     </row>
     <row r="28" spans="1:9" ht="13" customHeight="1">
       <c r="A28" s="6" t="s">
-        <v>17</v>
+        <v>75</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>53</v>
@@ -1638,9 +1885,11 @@
       </c>
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
-      <c r="I28" s="15"/>
-    </row>
-    <row r="29" spans="1:9" ht="13" customHeight="1">
+      <c r="I28" s="13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="46" customHeight="1">
       <c r="A29" s="6" t="s">
         <v>17</v>
       </c>
@@ -1648,10 +1897,10 @@
         <v>21</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>53</v>
@@ -1659,9 +1908,15 @@
       <c r="F29" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6"/>
-      <c r="I29" s="15"/>
+      <c r="G29" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="I29" s="13" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="30" spans="1:9" ht="13" customHeight="1">
       <c r="A30" s="6" t="s">
@@ -1671,55 +1926,47 @@
         <v>21</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>37</v>
+        <v>78</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G30" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I30" s="15"/>
+        <v>53</v>
+      </c>
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+      <c r="I30" s="13" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="31" spans="1:9" ht="13" customHeight="1">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C31" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E31" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="I31" s="15" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" ht="13" customHeight="1">
+      <c r="C31" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="13"/>
+    </row>
+    <row r="32" spans="1:9" ht="31" customHeight="1">
       <c r="A32" s="6" t="s">
         <v>17</v>
       </c>
@@ -1727,24 +1974,26 @@
         <v>21</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>1</v>
+        <v>53</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>9</v>
+        <v>53</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I32" s="15"/>
+        <v>73</v>
+      </c>
+      <c r="I32" s="13" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="33" spans="1:9" ht="13" customHeight="1">
       <c r="A33" s="6" t="s">
@@ -1754,16 +2003,16 @@
         <v>21</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G33" s="6" t="s">
         <v>0</v>
@@ -1771,34 +2020,36 @@
       <c r="H33" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I33" s="15"/>
+      <c r="I33" s="13"/>
     </row>
     <row r="34" spans="1:9" ht="13" customHeight="1">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C34" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E34" s="6" t="s">
+      <c r="C34" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G34" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="F34" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G34" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H34" s="6" t="s">
+      <c r="H34" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="I34" s="15"/>
+      <c r="I34" s="13" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="35" spans="1:9" ht="13" customHeight="1">
       <c r="A35" s="6" t="s">
@@ -1808,80 +2059,78 @@
         <v>21</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>92</v>
+        <v>39</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>92</v>
+        <v>39</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>74</v>
+        <v>9</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="I35" s="15" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="14">
-      <c r="A36" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="I35" s="13"/>
+    </row>
+    <row r="36" spans="1:9" ht="13" customHeight="1">
+      <c r="A36" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E36" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="F36" s="7" t="s">
+      <c r="H36" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I36" s="13"/>
+    </row>
+    <row r="37" spans="1:9" ht="13" customHeight="1">
+      <c r="A37" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F37" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G36" s="7" t="s">
+      <c r="G37" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="H36" s="7" t="s">
+      <c r="H37" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I36" s="15"/>
-    </row>
-    <row r="37" spans="1:9" ht="13" customHeight="1">
-      <c r="A37" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="E37" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="F37" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G37" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="H37" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="I37" s="15"/>
+      <c r="I37" s="13"/>
     </row>
     <row r="38" spans="1:9" ht="13" customHeight="1">
       <c r="A38" s="6" t="s">
@@ -1891,122 +2140,126 @@
         <v>21</v>
       </c>
       <c r="C38" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="I38" s="13" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="14">
+      <c r="A39" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="I39" s="13"/>
+    </row>
+    <row r="40" spans="1:9" ht="13" customHeight="1">
+      <c r="A40" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="I40" s="13"/>
+    </row>
+    <row r="41" spans="1:9" ht="13" customHeight="1">
+      <c r="A41" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C41" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D41" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="E41" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="F38" s="6" t="s">
+      <c r="F41" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G38" s="6" t="s">
+      <c r="G41" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="H38" s="6" t="s">
+      <c r="H41" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I38" s="15"/>
-    </row>
-    <row r="39" spans="1:9" ht="13" customHeight="1">
-      <c r="A39" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C39" s="6" t="s">
+      <c r="I41" s="13"/>
+    </row>
+    <row r="42" spans="1:9" ht="13" customHeight="1">
+      <c r="A42" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="D42" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="E39" s="6" t="s">
+      <c r="E42" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="F39" s="6" t="s">
+      <c r="F42" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="G39" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H39" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I39" s="15"/>
-    </row>
-    <row r="40" spans="1:9" ht="13" customHeight="1">
-      <c r="A40" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="G40" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I40" s="15"/>
-    </row>
-    <row r="41" spans="1:9" ht="15">
-      <c r="A41" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C41" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="E41" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="G41" s="7"/>
-      <c r="H41" s="7"/>
-      <c r="I41" s="15" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="30">
-      <c r="A42" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B42" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D42" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="E42" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>53</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>0</v>
@@ -2014,28 +2267,26 @@
       <c r="H42" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I42" s="15" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="30">
-      <c r="A43" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B43" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D43" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>53</v>
+      <c r="I42" s="13"/>
+    </row>
+    <row r="43" spans="1:9" ht="13" customHeight="1">
+      <c r="A43" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>6</v>
       </c>
       <c r="G43" s="6" t="s">
         <v>0</v>
@@ -2043,22 +2294,20 @@
       <c r="H43" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I43" s="15" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="30">
-      <c r="A44" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B44" s="7" t="s">
+      <c r="I43" s="13"/>
+    </row>
+    <row r="44" spans="1:9" ht="15">
+      <c r="A44" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B44" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E44" s="7" t="s">
         <v>53</v>
@@ -2066,88 +2315,144 @@
       <c r="F44" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="G44" s="7" t="s">
+      <c r="G44" s="7"/>
+      <c r="H44" s="7"/>
+      <c r="I44" s="13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="30">
+      <c r="A45" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I45" s="13" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="30">
+      <c r="A46" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I46" s="13" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="30">
+      <c r="A47" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H47" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="H44" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="I44" s="15" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" ht="14">
-      <c r="A45" s="7"/>
-      <c r="B45" s="7"/>
-      <c r="C45" s="13"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="7"/>
-      <c r="F45" s="7"/>
-      <c r="G45" s="7"/>
-      <c r="H45" s="7"/>
-      <c r="I45" s="15"/>
-    </row>
-    <row r="46" spans="1:9" ht="14">
-      <c r="A46" s="7"/>
-      <c r="B46" s="7"/>
-      <c r="C46" s="7"/>
-      <c r="D46" s="7"/>
-      <c r="E46" s="7"/>
-      <c r="F46" s="7"/>
-      <c r="G46" s="7"/>
-      <c r="H46" s="7"/>
-      <c r="I46" s="15"/>
-    </row>
-    <row r="47" spans="1:9" ht="14">
-      <c r="A47" s="7"/>
-      <c r="B47" s="7"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="7"/>
-      <c r="F47" s="7"/>
-      <c r="G47" s="7"/>
-      <c r="H47" s="7"/>
-      <c r="I47" s="15"/>
+      <c r="I47" s="13" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="48" spans="1:9" ht="14">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
-      <c r="C48" s="7"/>
-      <c r="D48" s="7"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="11"/>
       <c r="E48" s="7"/>
       <c r="F48" s="7"/>
       <c r="G48" s="7"/>
       <c r="H48" s="7"/>
-      <c r="I48" s="15"/>
-    </row>
-    <row r="49" spans="1:7">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
-    </row>
-    <row r="50" spans="1:7">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="5"/>
-      <c r="D50" s="5"/>
-      <c r="E50" s="5"/>
-      <c r="F50" s="5"/>
-      <c r="G50" s="5"/>
-    </row>
-    <row r="51" spans="1:7">
-      <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-      <c r="G51" s="5"/>
-    </row>
-    <row r="52" spans="1:7">
+      <c r="I48" s="13"/>
+    </row>
+    <row r="49" spans="1:9" ht="14">
+      <c r="A49" s="7"/>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="13"/>
+    </row>
+    <row r="50" spans="1:9" ht="14">
+      <c r="A50" s="7"/>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="7"/>
+      <c r="I50" s="13"/>
+    </row>
+    <row r="51" spans="1:9" ht="14">
+      <c r="A51" s="7"/>
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="13"/>
+    </row>
+    <row r="52" spans="1:9">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="5"/>
@@ -2156,7 +2461,7 @@
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
     </row>
-    <row r="53" spans="1:7">
+    <row r="53" spans="1:9">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="5"/>
@@ -2165,7 +2470,7 @@
       <c r="F53" s="5"/>
       <c r="G53" s="5"/>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:9">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="5"/>
@@ -2174,113 +2479,124 @@
       <c r="F54" s="5"/>
       <c r="G54" s="5"/>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:9">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
-    </row>
-    <row r="56" spans="1:7">
+      <c r="C55" s="5"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
+    </row>
+    <row r="56" spans="1:9">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
-    </row>
-    <row r="57" spans="1:7">
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+    </row>
+    <row r="57" spans="1:9">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
-    </row>
-    <row r="58" spans="1:7">
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+      <c r="G57" s="5"/>
+    </row>
+    <row r="58" spans="1:9">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
     </row>
-    <row r="59" spans="1:7">
+    <row r="59" spans="1:9">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
     </row>
-    <row r="60" spans="1:7">
+    <row r="60" spans="1:9">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
     </row>
-    <row r="61" spans="1:7">
+    <row r="61" spans="1:9">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
     </row>
-    <row r="62" spans="1:7">
+    <row r="62" spans="1:9">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
     </row>
-    <row r="63" spans="1:7">
+    <row r="63" spans="1:9">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
     </row>
-    <row r="64" spans="1:7">
+    <row r="64" spans="1:9">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
     </row>
-    <row r="65" spans="1:8">
+    <row r="65" spans="1:4">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
     </row>
-    <row r="66" spans="1:8">
+    <row r="66" spans="1:4">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
     </row>
-    <row r="67" spans="1:8">
+    <row r="67" spans="1:4">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
     </row>
-    <row r="68" spans="1:8">
+    <row r="68" spans="1:4">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
     </row>
-    <row r="69" spans="1:8" ht="14">
+    <row r="69" spans="1:4">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-    </row>
-    <row r="70" spans="1:8">
+    </row>
+    <row r="70" spans="1:4">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
     </row>
-    <row r="71" spans="1:8">
+    <row r="71" spans="1:4">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
     </row>
-    <row r="72" spans="1:8">
+    <row r="72" spans="1:4" ht="14">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
-    </row>
-    <row r="73" spans="1:8">
+      <c r="C72" s="2"/>
+      <c r="D72" s="2"/>
+    </row>
+    <row r="73" spans="1:4">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
     </row>
-    <row r="74" spans="1:8">
+    <row r="74" spans="1:4">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
     </row>
-    <row r="75" spans="1:8">
+    <row r="75" spans="1:4">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
     </row>
-    <row r="76" spans="1:8">
+    <row r="76" spans="1:4">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
     </row>
-    <row r="77" spans="1:8">
+    <row r="77" spans="1:4">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
     </row>
-    <row r="78" spans="1:8">
+    <row r="78" spans="1:4">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
     </row>
-    <row r="79" spans="1:8" ht="14">
+    <row r="79" spans="1:4">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
-      <c r="E79" s="2"/>
-      <c r="F79" s="2"/>
-      <c r="G79" s="2"/>
-      <c r="H79" s="2"/>
-    </row>
-    <row r="80" spans="1:8">
+    </row>
+    <row r="80" spans="1:4">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
     </row>
@@ -2288,9 +2604,13 @@
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
     </row>
-    <row r="82" spans="1:8">
+    <row r="82" spans="1:8" ht="14">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
+      <c r="E82" s="2"/>
+      <c r="F82" s="2"/>
+      <c r="G82" s="2"/>
+      <c r="H82" s="2"/>
     </row>
     <row r="83" spans="1:8">
       <c r="A83" s="3"/>
@@ -2316,35 +2636,35 @@
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
     </row>
-    <row r="89" spans="1:8" ht="14">
+    <row r="89" spans="1:8">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
-      <c r="E89" s="2"/>
-      <c r="F89" s="2"/>
-      <c r="G89" s="2"/>
-      <c r="H89" s="2"/>
     </row>
     <row r="90" spans="1:8">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
     </row>
-    <row r="91" spans="1:8" ht="14">
+    <row r="91" spans="1:8">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
-      <c r="C91" s="2"/>
-      <c r="D91" s="2"/>
-    </row>
-    <row r="92" spans="1:8">
+    </row>
+    <row r="92" spans="1:8" ht="14">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
+      <c r="E92" s="2"/>
+      <c r="F92" s="2"/>
+      <c r="G92" s="2"/>
+      <c r="H92" s="2"/>
     </row>
     <row r="93" spans="1:8">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
     </row>
-    <row r="94" spans="1:8">
+    <row r="94" spans="1:8" ht="14">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
+      <c r="C94" s="2"/>
+      <c r="D94" s="2"/>
     </row>
     <row r="95" spans="1:8">
       <c r="A95" s="3"/>
@@ -2358,35 +2678,35 @@
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
     </row>
-    <row r="98" spans="1:4" ht="14">
+    <row r="98" spans="1:4">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
-      <c r="C98" s="4"/>
-      <c r="D98" s="4"/>
-    </row>
-    <row r="99" spans="1:4" ht="14">
+    </row>
+    <row r="99" spans="1:4">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
-      <c r="C99" s="2"/>
-      <c r="D99" s="2"/>
-    </row>
-    <row r="100" spans="1:4" ht="14">
+    </row>
+    <row r="100" spans="1:4">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
-      <c r="C100" s="2"/>
-      <c r="D100" s="2"/>
-    </row>
-    <row r="101" spans="1:4">
+    </row>
+    <row r="101" spans="1:4" ht="14">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
-    </row>
-    <row r="102" spans="1:4">
+      <c r="C101" s="4"/>
+      <c r="D101" s="4"/>
+    </row>
+    <row r="102" spans="1:4" ht="14">
       <c r="A102" s="3"/>
       <c r="B102" s="3"/>
-    </row>
-    <row r="103" spans="1:4">
+      <c r="C102" s="2"/>
+      <c r="D102" s="2"/>
+    </row>
+    <row r="103" spans="1:4" ht="14">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
+      <c r="C103" s="2"/>
+      <c r="D103" s="2"/>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="3"/>
@@ -2492,11 +2812,9 @@
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
     </row>
-    <row r="130" spans="1:8" ht="14">
+    <row r="130" spans="1:8">
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
-      <c r="C130" s="2"/>
-      <c r="D130" s="2"/>
     </row>
     <row r="131" spans="1:8">
       <c r="A131" s="3"/>
@@ -2506,9 +2824,11 @@
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
     </row>
-    <row r="133" spans="1:8">
+    <row r="133" spans="1:8" ht="14">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
+      <c r="C133" s="2"/>
+      <c r="D133" s="2"/>
     </row>
     <row r="134" spans="1:8">
       <c r="A134" s="3"/>
@@ -2526,39 +2846,39 @@
       <c r="A137" s="3"/>
       <c r="B137" s="3"/>
     </row>
-    <row r="138" spans="1:8" ht="14">
+    <row r="138" spans="1:8">
       <c r="A138" s="3"/>
       <c r="B138" s="3"/>
-      <c r="E138" s="4"/>
-      <c r="F138" s="4"/>
-      <c r="G138" s="4"/>
-      <c r="H138" s="4"/>
-    </row>
-    <row r="139" spans="1:8" ht="14">
+    </row>
+    <row r="139" spans="1:8">
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
-      <c r="E139" s="2"/>
-      <c r="F139" s="2"/>
-      <c r="G139" s="2"/>
-      <c r="H139" s="2"/>
-    </row>
-    <row r="140" spans="1:8" ht="14">
+    </row>
+    <row r="140" spans="1:8">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
-      <c r="C140" s="2"/>
-      <c r="D140" s="2"/>
-    </row>
-    <row r="141" spans="1:8">
+    </row>
+    <row r="141" spans="1:8" ht="14">
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
-    </row>
-    <row r="142" spans="1:8">
+      <c r="E141" s="4"/>
+      <c r="F141" s="4"/>
+      <c r="G141" s="4"/>
+      <c r="H141" s="4"/>
+    </row>
+    <row r="142" spans="1:8" ht="14">
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
-    </row>
-    <row r="143" spans="1:8">
+      <c r="E142" s="2"/>
+      <c r="F142" s="2"/>
+      <c r="G142" s="2"/>
+      <c r="H142" s="2"/>
+    </row>
+    <row r="143" spans="1:8" ht="14">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
+      <c r="C143" s="2"/>
+      <c r="D143" s="2"/>
     </row>
     <row r="144" spans="1:8">
       <c r="A144" s="3"/>
@@ -2584,13 +2904,9 @@
       <c r="A149" s="3"/>
       <c r="B149" s="3"/>
     </row>
-    <row r="150" spans="1:8" ht="14">
+    <row r="150" spans="1:8">
       <c r="A150" s="3"/>
       <c r="B150" s="3"/>
-      <c r="E150" s="2"/>
-      <c r="F150" s="2"/>
-      <c r="G150" s="2"/>
-      <c r="H150" s="2"/>
     </row>
     <row r="151" spans="1:8">
       <c r="A151" s="3"/>
@@ -2616,9 +2932,13 @@
       <c r="A155" s="3"/>
       <c r="B155" s="3"/>
     </row>
-    <row r="156" spans="1:8">
+    <row r="156" spans="1:8" ht="14">
       <c r="A156" s="3"/>
       <c r="B156" s="3"/>
+      <c r="E156" s="2"/>
+      <c r="F156" s="2"/>
+      <c r="G156" s="2"/>
+      <c r="H156" s="2"/>
     </row>
     <row r="157" spans="1:8">
       <c r="A157" s="3"/>
@@ -2748,29 +3068,29 @@
       <c r="A188" s="3"/>
       <c r="B188" s="3"/>
     </row>
-    <row r="189" spans="1:4" ht="14">
+    <row r="189" spans="1:4">
       <c r="A189" s="3"/>
       <c r="B189" s="3"/>
-      <c r="C189" s="4"/>
-      <c r="D189" s="4"/>
-    </row>
-    <row r="190" spans="1:4" ht="14">
+    </row>
+    <row r="190" spans="1:4">
       <c r="A190" s="3"/>
       <c r="B190" s="3"/>
-      <c r="C190" s="2"/>
-      <c r="D190" s="2"/>
     </row>
     <row r="191" spans="1:4">
       <c r="A191" s="3"/>
       <c r="B191" s="3"/>
     </row>
-    <row r="192" spans="1:4">
+    <row r="192" spans="1:4" ht="14">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
-    </row>
-    <row r="193" spans="1:4">
+      <c r="C192" s="4"/>
+      <c r="D192" s="4"/>
+    </row>
+    <row r="193" spans="1:4" ht="14">
       <c r="A193" s="3"/>
       <c r="B193" s="3"/>
+      <c r="C193" s="2"/>
+      <c r="D193" s="2"/>
     </row>
     <row r="194" spans="1:4">
       <c r="A194" s="3"/>
@@ -2800,11 +3120,9 @@
       <c r="A200" s="3"/>
       <c r="B200" s="3"/>
     </row>
-    <row r="201" spans="1:4" ht="14">
+    <row r="201" spans="1:4">
       <c r="A201" s="3"/>
       <c r="B201" s="3"/>
-      <c r="C201" s="2"/>
-      <c r="D201" s="2"/>
     </row>
     <row r="202" spans="1:4">
       <c r="A202" s="3"/>
@@ -2828,9 +3146,11 @@
       <c r="A206" s="3"/>
       <c r="B206" s="3"/>
     </row>
-    <row r="207" spans="1:4">
+    <row r="207" spans="1:4" ht="14">
       <c r="A207" s="3"/>
       <c r="B207" s="3"/>
+      <c r="C207" s="2"/>
+      <c r="D207" s="2"/>
     </row>
     <row r="208" spans="1:4">
       <c r="A208" s="3"/>
@@ -2859,20 +3179,14 @@
     <row r="214" spans="1:4">
       <c r="A214" s="3"/>
       <c r="B214" s="3"/>
-      <c r="C214" s="3"/>
-      <c r="D214" s="3"/>
     </row>
     <row r="215" spans="1:4">
       <c r="A215" s="3"/>
       <c r="B215" s="3"/>
-      <c r="C215" s="3"/>
-      <c r="D215" s="3"/>
     </row>
     <row r="216" spans="1:4">
       <c r="A216" s="3"/>
       <c r="B216" s="3"/>
-      <c r="C216" s="3"/>
-      <c r="D216" s="3"/>
     </row>
     <row r="217" spans="1:4">
       <c r="A217" s="3"/>
@@ -2893,14 +3207,20 @@
       <c r="D219" s="3"/>
     </row>
     <row r="220" spans="1:4">
+      <c r="A220" s="3"/>
+      <c r="B220" s="3"/>
       <c r="C220" s="3"/>
       <c r="D220" s="3"/>
     </row>
     <row r="221" spans="1:4">
+      <c r="A221" s="3"/>
+      <c r="B221" s="3"/>
       <c r="C221" s="3"/>
       <c r="D221" s="3"/>
     </row>
     <row r="222" spans="1:4">
+      <c r="A222" s="3"/>
+      <c r="B222" s="3"/>
       <c r="C222" s="3"/>
       <c r="D222" s="3"/>
     </row>
@@ -3648,10 +3968,22 @@
       <c r="C408" s="3"/>
       <c r="D408" s="3"/>
     </row>
+    <row r="409" spans="3:4">
+      <c r="C409" s="3"/>
+      <c r="D409" s="3"/>
+    </row>
+    <row r="410" spans="3:4">
+      <c r="C410" s="3"/>
+      <c r="D410" s="3"/>
+    </row>
+    <row r="411" spans="3:4">
+      <c r="C411" s="3"/>
+      <c r="D411" s="3"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F39" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C45:C68">
-    <sortCondition ref="C45:C68"/>
+  <autoFilter ref="A1:F42" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C48:C71">
+    <sortCondition ref="C48:C71"/>
   </sortState>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.74791666666666667" right="0.74791666666666667" top="0.98402777777777772" bottom="0.98402777777777772" header="0.51180555555555551" footer="0.51180555555555551"/>

</xml_diff>